<commit_message>
chore: aggiornamento automatico dati fantacalcio 2026-09-14
</commit_message>
<xml_diff>
--- a/export/lista_asta.xlsx
+++ b/export/lista_asta.xlsx
@@ -704,10 +704,10 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T2" t="n">
-        <v>6.17</v>
+        <v>5.75</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -791,10 +791,10 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T3" t="n">
-        <v>5.33</v>
+        <v>5.12</v>
       </c>
       <c r="U3" t="n">
         <v>0</v>
@@ -1030,10 +1030,10 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T6" t="n">
-        <v>5.83</v>
+        <v>5.12</v>
       </c>
       <c r="U6" t="n">
         <v>0</v>
@@ -1374,10 +1374,10 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T10" t="n">
-        <v>4.5</v>
+        <v>4.25</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
@@ -1461,10 +1461,10 @@
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T11" t="n">
-        <v>6</v>
+        <v>5.62</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
@@ -1635,10 +1635,10 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T13" t="n">
-        <v>6</v>
+        <v>5.88</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
@@ -1931,10 +1931,10 @@
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T17" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U17" t="n">
         <v>0</v>
@@ -2016,10 +2016,10 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T18" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U18" t="n">
         <v>0</v>
@@ -2275,10 +2275,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T21" t="n">
-        <v>4.33</v>
+        <v>4.12</v>
       </c>
       <c r="U21" t="n">
         <v>0</v>
@@ -2447,10 +2447,10 @@
         <v>0</v>
       </c>
       <c r="S23" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T23" t="n">
-        <v>3.17</v>
+        <v>3.75</v>
       </c>
       <c r="U23" t="n">
         <v>0</v>
@@ -2706,10 +2706,10 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T26" t="n">
-        <v>5.17</v>
+        <v>5.38</v>
       </c>
       <c r="U26" t="n">
         <v>0</v>
@@ -3004,10 +3004,10 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T30" t="n">
-        <v>3.25</v>
+        <v>2.83</v>
       </c>
       <c r="U30" t="n">
         <v>0</v>
@@ -6131,10 +6131,10 @@
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T5" t="n">
-        <v>7.67</v>
+        <v>7</v>
       </c>
       <c r="U5" t="n">
         <v>1</v>
@@ -6218,10 +6218,10 @@
         <v>0</v>
       </c>
       <c r="S6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T6" t="n">
-        <v>6.5</v>
+        <v>6.12</v>
       </c>
       <c r="U6" t="n">
         <v>0</v>
@@ -6305,10 +6305,10 @@
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T7" t="n">
-        <v>6.33</v>
+        <v>6.38</v>
       </c>
       <c r="U7" t="n">
         <v>0</v>
@@ -6453,10 +6453,10 @@
         <v>0</v>
       </c>
       <c r="S9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T9" t="n">
-        <v>6</v>
+        <v>5.75</v>
       </c>
       <c r="U9" t="n">
         <v>0</v>
@@ -6540,10 +6540,10 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T10" t="n">
-        <v>5.67</v>
+        <v>5.88</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
@@ -6801,10 +6801,10 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T13" t="n">
-        <v>6.17</v>
+        <v>6.12</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
@@ -6975,10 +6975,10 @@
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T15" t="n">
-        <v>6.17</v>
+        <v>6</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -7062,10 +7062,10 @@
         <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T16" t="n">
-        <v>5.33</v>
+        <v>5.5</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
@@ -7408,13 +7408,13 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T20" t="n">
-        <v>5.5</v>
+        <v>6.12</v>
       </c>
       <c r="U20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V20" t="n">
         <v>0</v>
@@ -7495,10 +7495,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T21" t="n">
-        <v>6.75</v>
+        <v>6.33</v>
       </c>
       <c r="U21" t="n">
         <v>0</v>
@@ -7928,13 +7928,13 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T26" t="n">
-        <v>6.67</v>
+        <v>7.5</v>
       </c>
       <c r="U26" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V26" t="n">
         <v>0</v>
@@ -8187,10 +8187,10 @@
         <v>0</v>
       </c>
       <c r="S29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T29" t="n">
-        <v>6.5</v>
+        <v>6.25</v>
       </c>
       <c r="U29" t="n">
         <v>0</v>
@@ -8274,10 +8274,10 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T30" t="n">
-        <v>7</v>
+        <v>6.67</v>
       </c>
       <c r="U30" t="n">
         <v>0</v>
@@ -8361,10 +8361,10 @@
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T31" t="n">
-        <v>6.5</v>
+        <v>6.12</v>
       </c>
       <c r="U31" t="n">
         <v>0</v>
@@ -9319,10 +9319,10 @@
         <v>0</v>
       </c>
       <c r="S43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T43" t="n">
-        <v>6</v>
+        <v>5.83</v>
       </c>
       <c r="U43" t="n">
         <v>0</v>
@@ -9580,7 +9580,7 @@
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T46" t="n">
         <v>6</v>
@@ -9926,10 +9926,10 @@
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T50" t="n">
-        <v>5.67</v>
+        <v>5.62</v>
       </c>
       <c r="U50" t="n">
         <v>0</v>
@@ -10274,10 +10274,10 @@
         <v>0</v>
       </c>
       <c r="S54" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T54" t="n">
-        <v>5</v>
+        <v>5.25</v>
       </c>
       <c r="U54" t="n">
         <v>0</v>
@@ -10359,10 +10359,10 @@
         <v>0</v>
       </c>
       <c r="S55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T55" t="n">
-        <v>5.5</v>
+        <v>5.75</v>
       </c>
       <c r="U55" t="n">
         <v>0</v>
@@ -10707,10 +10707,10 @@
         <v>0</v>
       </c>
       <c r="S59" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T59" t="n">
-        <v>5.75</v>
+        <v>6</v>
       </c>
       <c r="U59" t="n">
         <v>0</v>
@@ -10794,10 +10794,10 @@
         <v>0</v>
       </c>
       <c r="S60" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T60" t="n">
-        <v>5.75</v>
+        <v>5.67</v>
       </c>
       <c r="U60" t="n">
         <v>0</v>
@@ -10968,7 +10968,7 @@
         <v>0</v>
       </c>
       <c r="S62" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T62" t="n">
         <v>6</v>
@@ -11142,10 +11142,10 @@
         <v>0</v>
       </c>
       <c r="S64" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T64" t="n">
-        <v>5.33</v>
+        <v>5.38</v>
       </c>
       <c r="U64" t="n">
         <v>0</v>
@@ -11227,10 +11227,10 @@
         <v>0</v>
       </c>
       <c r="S65" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T65" t="n">
-        <v>5.67</v>
+        <v>5.5</v>
       </c>
       <c r="U65" t="n">
         <v>0</v>
@@ -11314,10 +11314,10 @@
         <v>0</v>
       </c>
       <c r="S66" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T66" t="n">
-        <v>5.67</v>
+        <v>5.75</v>
       </c>
       <c r="U66" t="n">
         <v>0</v>
@@ -11399,10 +11399,10 @@
         <v>0</v>
       </c>
       <c r="S67" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T67" t="n">
-        <v>5.17</v>
+        <v>5.5</v>
       </c>
       <c r="U67" t="n">
         <v>0</v>
@@ -11484,10 +11484,10 @@
         <v>0</v>
       </c>
       <c r="S68" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T68" t="n">
-        <v>6.17</v>
+        <v>6.25</v>
       </c>
       <c r="U68" t="n">
         <v>0</v>
@@ -11741,10 +11741,10 @@
         <v>0</v>
       </c>
       <c r="S71" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T71" t="n">
-        <v>5.83</v>
+        <v>6.12</v>
       </c>
       <c r="U71" t="n">
         <v>0</v>
@@ -11891,10 +11891,10 @@
       <c r="Q73" t="inlineStr"/>
       <c r="R73" t="inlineStr"/>
       <c r="S73" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T73" t="n">
-        <v>7.67</v>
+        <v>7.12</v>
       </c>
       <c r="U73" t="n">
         <v>1</v>
@@ -12074,10 +12074,10 @@
       <c r="Q76" t="inlineStr"/>
       <c r="R76" t="inlineStr"/>
       <c r="S76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T76" t="n">
-        <v>5.5</v>
+        <v>5.75</v>
       </c>
       <c r="U76" t="n">
         <v>0</v>
@@ -12135,13 +12135,13 @@
       <c r="Q77" t="inlineStr"/>
       <c r="R77" t="inlineStr"/>
       <c r="S77" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T77" t="n">
-        <v>6.67</v>
+        <v>7.5</v>
       </c>
       <c r="U77" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V77" t="n">
         <v>2</v>
@@ -12257,10 +12257,10 @@
       <c r="Q79" t="inlineStr"/>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T79" t="n">
-        <v>6.17</v>
+        <v>6.12</v>
       </c>
       <c r="U79" t="n">
         <v>0</v>
@@ -12440,10 +12440,10 @@
       <c r="Q82" t="inlineStr"/>
       <c r="R82" t="inlineStr"/>
       <c r="S82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T82" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U82" t="n">
         <v>0</v>
@@ -12501,10 +12501,10 @@
       <c r="Q83" t="inlineStr"/>
       <c r="R83" t="inlineStr"/>
       <c r="S83" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T83" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U83" t="n">
         <v>0</v>
@@ -12852,16 +12852,16 @@
         <v>0</v>
       </c>
       <c r="S88" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T88" t="n">
-        <v>5.83</v>
+        <v>6.12</v>
       </c>
       <c r="U88" t="n">
         <v>0</v>
       </c>
       <c r="V88" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W88" t="n">
         <v>2</v>
@@ -13461,10 +13461,10 @@
         <v>0</v>
       </c>
       <c r="S95" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T95" t="n">
-        <v>5.75</v>
+        <v>5.5</v>
       </c>
       <c r="U95" t="n">
         <v>0</v>
@@ -13548,10 +13548,10 @@
         <v>0</v>
       </c>
       <c r="S96" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T96" t="n">
-        <v>5.5</v>
+        <v>5.83</v>
       </c>
       <c r="U96" t="n">
         <v>0</v>
@@ -13722,7 +13722,7 @@
         <v>0</v>
       </c>
       <c r="S98" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T98" t="n">
         <v>5.5</v>
@@ -14155,10 +14155,10 @@
         <v>0</v>
       </c>
       <c r="S103" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T103" t="n">
-        <v>5.67</v>
+        <v>5.5</v>
       </c>
       <c r="U103" t="n">
         <v>0</v>
@@ -14242,10 +14242,10 @@
         <v>0</v>
       </c>
       <c r="S104" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T104" t="n">
-        <v>6.17</v>
+        <v>5.75</v>
       </c>
       <c r="U104" t="n">
         <v>0</v>
@@ -14501,10 +14501,10 @@
         <v>0</v>
       </c>
       <c r="S107" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T107" t="n">
-        <v>5.67</v>
+        <v>5.62</v>
       </c>
       <c r="U107" t="n">
         <v>0</v>
@@ -14932,10 +14932,10 @@
         <v>0</v>
       </c>
       <c r="S112" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T112" t="n">
-        <v>5.33</v>
+        <v>5.5</v>
       </c>
       <c r="U112" t="n">
         <v>0</v>
@@ -15019,10 +15019,10 @@
         <v>0</v>
       </c>
       <c r="S113" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T113" t="n">
-        <v>7.17</v>
+        <v>7</v>
       </c>
       <c r="U113" t="n">
         <v>1</v>
@@ -15189,10 +15189,10 @@
         <v>0</v>
       </c>
       <c r="S115" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T115" t="n">
-        <v>5.75</v>
+        <v>5.5</v>
       </c>
       <c r="U115" t="n">
         <v>0</v>
@@ -15361,10 +15361,10 @@
         <v>0</v>
       </c>
       <c r="S117" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T117" t="n">
-        <v>5.83</v>
+        <v>5.75</v>
       </c>
       <c r="U117" t="n">
         <v>0</v>
@@ -15881,16 +15881,16 @@
         <v>0</v>
       </c>
       <c r="S123" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T123" t="n">
-        <v>5.83</v>
+        <v>6.12</v>
       </c>
       <c r="U123" t="n">
         <v>0</v>
       </c>
       <c r="V123" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W123" t="n">
         <v>9</v>
@@ -15966,10 +15966,10 @@
         <v>0</v>
       </c>
       <c r="S124" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T124" t="n">
-        <v>6.67</v>
+        <v>6.5</v>
       </c>
       <c r="U124" t="n">
         <v>0</v>
@@ -16138,10 +16138,10 @@
         <v>0</v>
       </c>
       <c r="S126" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T126" t="n">
-        <v>5.83</v>
+        <v>5.62</v>
       </c>
       <c r="U126" t="n">
         <v>0</v>
@@ -16393,10 +16393,10 @@
         <v>0</v>
       </c>
       <c r="S129" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T129" t="n">
-        <v>5.33</v>
+        <v>5.25</v>
       </c>
       <c r="U129" t="n">
         <v>0</v>
@@ -16691,10 +16691,10 @@
       <c r="Q133" t="inlineStr"/>
       <c r="R133" t="inlineStr"/>
       <c r="S133" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T133" t="n">
-        <v>6.5</v>
+        <v>6.38</v>
       </c>
       <c r="U133" t="n">
         <v>0</v>
@@ -17179,16 +17179,16 @@
       <c r="Q141" t="inlineStr"/>
       <c r="R141" t="inlineStr"/>
       <c r="S141" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T141" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="U141" t="n">
         <v>0</v>
       </c>
       <c r="V141" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W141" t="inlineStr"/>
       <c r="X141" t="inlineStr"/>
@@ -18594,10 +18594,10 @@
         <v>0</v>
       </c>
       <c r="S158" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T158" t="n">
-        <v>5.17</v>
+        <v>5.38</v>
       </c>
       <c r="U158" t="n">
         <v>0</v>
@@ -19752,10 +19752,10 @@
       <c r="Q172" t="inlineStr"/>
       <c r="R172" t="inlineStr"/>
       <c r="S172" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T172" t="n">
-        <v>6.33</v>
+        <v>6.25</v>
       </c>
       <c r="U172" t="n">
         <v>0</v>
@@ -20240,10 +20240,10 @@
       <c r="Q180" t="inlineStr"/>
       <c r="R180" t="inlineStr"/>
       <c r="S180" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T180" t="n">
-        <v>6</v>
+        <v>5.75</v>
       </c>
       <c r="U180" t="n">
         <v>0</v>
@@ -21412,16 +21412,16 @@
         <v>1</v>
       </c>
       <c r="S3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T3" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="U3" t="n">
         <v>0</v>
       </c>
       <c r="V3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W3" t="n">
         <v>0</v>
@@ -21760,7 +21760,7 @@
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T7" t="n">
         <v>7.5</v>
@@ -21769,7 +21769,7 @@
         <v>1</v>
       </c>
       <c r="V7" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W7" t="n">
         <v>4</v>
@@ -21930,10 +21930,10 @@
         <v>3</v>
       </c>
       <c r="S9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T9" t="n">
-        <v>8</v>
+        <v>7.62</v>
       </c>
       <c r="U9" t="n">
         <v>1</v>
@@ -22017,10 +22017,10 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T10" t="n">
-        <v>10.17</v>
+        <v>9.119999999999999</v>
       </c>
       <c r="U10" t="n">
         <v>3</v>
@@ -22278,10 +22278,10 @@
         <v>3</v>
       </c>
       <c r="S13" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T13" t="n">
-        <v>7</v>
+        <v>6.67</v>
       </c>
       <c r="U13" t="n">
         <v>1</v>
@@ -22452,10 +22452,10 @@
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T15" t="n">
-        <v>8.5</v>
+        <v>7.83</v>
       </c>
       <c r="U15" t="n">
         <v>1</v>
@@ -22626,10 +22626,10 @@
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T17" t="n">
-        <v>6.83</v>
+        <v>6.5</v>
       </c>
       <c r="U17" t="n">
         <v>0</v>
@@ -22974,10 +22974,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T21" t="n">
-        <v>6.67</v>
+        <v>6.38</v>
       </c>
       <c r="U21" t="n">
         <v>1</v>
@@ -23059,10 +23059,10 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T22" t="n">
-        <v>6</v>
+        <v>5.88</v>
       </c>
       <c r="U22" t="n">
         <v>0</v>
@@ -23231,7 +23231,7 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T24" t="n">
         <v>5.5</v>
@@ -23405,10 +23405,10 @@
         <v>1</v>
       </c>
       <c r="S26" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T26" t="n">
-        <v>7.17</v>
+        <v>6.75</v>
       </c>
       <c r="U26" t="n">
         <v>1</v>
@@ -23490,7 +23490,7 @@
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T27" t="n">
         <v>6</v>
@@ -23664,16 +23664,16 @@
         <v>1</v>
       </c>
       <c r="S29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T29" t="n">
-        <v>6.33</v>
+        <v>6.5</v>
       </c>
       <c r="U29" t="n">
         <v>0</v>
       </c>
       <c r="V29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W29" t="n">
         <v>6</v>
@@ -23751,10 +23751,10 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T30" t="n">
-        <v>7.33</v>
+        <v>6.75</v>
       </c>
       <c r="U30" t="n">
         <v>1</v>
@@ -23923,10 +23923,10 @@
         <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T32" t="n">
-        <v>8.33</v>
+        <v>7.62</v>
       </c>
       <c r="U32" t="n">
         <v>2</v>
@@ -24110,10 +24110,10 @@
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T35" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U35" t="n">
         <v>0</v>
@@ -24232,10 +24232,10 @@
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T37" t="n">
-        <v>5.5</v>
+        <v>5.67</v>
       </c>
       <c r="U37" t="n">
         <v>0</v>
@@ -24354,13 +24354,13 @@
       <c r="Q39" t="inlineStr"/>
       <c r="R39" t="inlineStr"/>
       <c r="S39" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T39" t="n">
-        <v>5</v>
+        <v>9.5</v>
       </c>
       <c r="U39" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V39" t="n">
         <v>0</v>
@@ -24953,10 +24953,10 @@
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T46" t="n">
-        <v>6</v>
+        <v>5.88</v>
       </c>
       <c r="U46" t="n">
         <v>0</v>
@@ -25038,10 +25038,10 @@
         <v>1</v>
       </c>
       <c r="S47" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T47" t="n">
-        <v>6.33</v>
+        <v>6.25</v>
       </c>
       <c r="U47" t="n">
         <v>0</v>
@@ -25125,10 +25125,10 @@
         <v>0</v>
       </c>
       <c r="S48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T48" t="n">
-        <v>5.67</v>
+        <v>5.62</v>
       </c>
       <c r="U48" t="n">
         <v>0</v>
@@ -25473,10 +25473,10 @@
         <v>0</v>
       </c>
       <c r="S52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T52" t="n">
-        <v>7.33</v>
+        <v>7</v>
       </c>
       <c r="U52" t="n">
         <v>0</v>
@@ -25560,10 +25560,10 @@
         <v>0</v>
       </c>
       <c r="S53" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T53" t="n">
-        <v>5.83</v>
+        <v>5.75</v>
       </c>
       <c r="U53" t="n">
         <v>0</v>
@@ -26169,10 +26169,10 @@
         <v>0</v>
       </c>
       <c r="S60" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T60" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U60" t="n">
         <v>0</v>
@@ -26256,13 +26256,13 @@
         <v>0</v>
       </c>
       <c r="S61" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T61" t="n">
-        <v>5.67</v>
+        <v>6.75</v>
       </c>
       <c r="U61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V61" t="n">
         <v>0</v>
@@ -26776,10 +26776,10 @@
         <v>0</v>
       </c>
       <c r="S67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T67" t="n">
-        <v>8.75</v>
+        <v>7.67</v>
       </c>
       <c r="U67" t="n">
         <v>1</v>
@@ -26950,10 +26950,10 @@
         <v>0</v>
       </c>
       <c r="S69" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T69" t="n">
-        <v>5.83</v>
+        <v>5.88</v>
       </c>
       <c r="U69" t="n">
         <v>0</v>
@@ -27035,10 +27035,10 @@
         <v>0</v>
       </c>
       <c r="S70" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T70" t="n">
-        <v>8.25</v>
+        <v>7.5</v>
       </c>
       <c r="U70" t="n">
         <v>1</v>
@@ -27122,10 +27122,10 @@
         <v>0</v>
       </c>
       <c r="S71" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T71" t="n">
-        <v>5.67</v>
+        <v>5.62</v>
       </c>
       <c r="U71" t="n">
         <v>0</v>
@@ -27209,10 +27209,10 @@
         <v>0</v>
       </c>
       <c r="S72" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T72" t="n">
-        <v>5.67</v>
+        <v>5.75</v>
       </c>
       <c r="U72" t="n">
         <v>0</v>
@@ -27296,10 +27296,10 @@
         <v>0</v>
       </c>
       <c r="S73" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T73" t="n">
-        <v>6</v>
+        <v>6.12</v>
       </c>
       <c r="U73" t="n">
         <v>0</v>
@@ -27383,13 +27383,13 @@
         <v>0</v>
       </c>
       <c r="S74" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T74" t="n">
-        <v>6.33</v>
+        <v>7.38</v>
       </c>
       <c r="U74" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V74" t="n">
         <v>0</v>
@@ -27470,10 +27470,10 @@
         <v>0</v>
       </c>
       <c r="S75" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T75" t="n">
-        <v>6.17</v>
+        <v>6</v>
       </c>
       <c r="U75" t="n">
         <v>0</v>
@@ -27881,10 +27881,10 @@
       <c r="Q80" t="inlineStr"/>
       <c r="R80" t="inlineStr"/>
       <c r="S80" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T80" t="n">
-        <v>7.5</v>
+        <v>7.38</v>
       </c>
       <c r="U80" t="n">
         <v>1</v>
@@ -27942,10 +27942,10 @@
       <c r="Q81" t="inlineStr"/>
       <c r="R81" t="inlineStr"/>
       <c r="S81" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T81" t="n">
-        <v>6.67</v>
+        <v>6.62</v>
       </c>
       <c r="U81" t="n">
         <v>0</v>
@@ -28003,16 +28003,16 @@
       <c r="Q82" t="inlineStr"/>
       <c r="R82" t="inlineStr"/>
       <c r="S82" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T82" t="n">
-        <v>5.5</v>
+        <v>6</v>
       </c>
       <c r="U82" t="n">
         <v>0</v>
       </c>
       <c r="V82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W82" t="inlineStr"/>
       <c r="X82" t="inlineStr"/>
@@ -28125,7 +28125,7 @@
       <c r="Q84" t="inlineStr"/>
       <c r="R84" t="inlineStr"/>
       <c r="S84" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T84" t="n">
         <v>5.5</v>
@@ -28186,10 +28186,10 @@
       <c r="Q85" t="inlineStr"/>
       <c r="R85" t="inlineStr"/>
       <c r="S85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T85" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U85" t="n">
         <v>0</v>
@@ -28391,7 +28391,7 @@
         <v>0</v>
       </c>
       <c r="S88" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T88" t="n">
         <v>5.5</v>
@@ -28565,10 +28565,10 @@
         <v>0</v>
       </c>
       <c r="S90" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T90" t="n">
-        <v>6.83</v>
+        <v>6.5</v>
       </c>
       <c r="U90" t="n">
         <v>1</v>
@@ -28998,10 +28998,10 @@
         <v>0</v>
       </c>
       <c r="S95" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T95" t="n">
-        <v>5.67</v>
+        <v>5.62</v>
       </c>
       <c r="U95" t="n">
         <v>0</v>
@@ -29085,13 +29085,13 @@
         <v>0</v>
       </c>
       <c r="S96" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T96" t="n">
-        <v>7.67</v>
+        <v>8.25</v>
       </c>
       <c r="U96" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V96" t="n">
         <v>1</v>
@@ -29172,13 +29172,13 @@
         <v>0</v>
       </c>
       <c r="S97" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T97" t="n">
-        <v>6.33</v>
+        <v>8.119999999999999</v>
       </c>
       <c r="U97" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V97" t="n">
         <v>1</v>
@@ -29259,7 +29259,7 @@
         <v>0</v>
       </c>
       <c r="S98" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T98" t="n">
         <v>6</v>
@@ -29433,7 +29433,7 @@
         <v>0</v>
       </c>
       <c r="S100" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T100" t="n">
         <v>6</v>
@@ -29520,10 +29520,10 @@
         <v>0</v>
       </c>
       <c r="S101" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T101" t="n">
-        <v>5.75</v>
+        <v>5.83</v>
       </c>
       <c r="U101" t="n">
         <v>0</v>
@@ -29781,10 +29781,10 @@
         <v>0</v>
       </c>
       <c r="S104" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T104" t="n">
-        <v>5.5</v>
+        <v>5.62</v>
       </c>
       <c r="U104" t="n">
         <v>0</v>
@@ -30040,10 +30040,10 @@
         <v>0</v>
       </c>
       <c r="S107" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T107" t="n">
-        <v>5.5</v>
+        <v>5.33</v>
       </c>
       <c r="U107" t="n">
         <v>0</v>
@@ -30212,10 +30212,10 @@
         <v>0</v>
       </c>
       <c r="S109" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T109" t="n">
-        <v>5.5</v>
+        <v>5.75</v>
       </c>
       <c r="U109" t="n">
         <v>0</v>
@@ -30384,16 +30384,16 @@
         <v>0</v>
       </c>
       <c r="S111" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T111" t="n">
-        <v>6.17</v>
+        <v>6.75</v>
       </c>
       <c r="U111" t="n">
         <v>0</v>
       </c>
       <c r="V111" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W111" t="n">
         <v>6</v>
@@ -30558,16 +30558,16 @@
         <v>0</v>
       </c>
       <c r="S113" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T113" t="n">
-        <v>6.5</v>
+        <v>6.75</v>
       </c>
       <c r="U113" t="n">
         <v>0</v>
       </c>
       <c r="V113" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W113" t="n">
         <v>4</v>
@@ -31335,10 +31335,10 @@
         <v>0</v>
       </c>
       <c r="S122" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T122" t="n">
-        <v>6.17</v>
+        <v>6.25</v>
       </c>
       <c r="U122" t="n">
         <v>0</v>
@@ -31420,16 +31420,16 @@
         <v>0</v>
       </c>
       <c r="S123" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T123" t="n">
-        <v>6</v>
+        <v>6.5</v>
       </c>
       <c r="U123" t="n">
         <v>0</v>
       </c>
       <c r="V123" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W123" t="n">
         <v>0</v>
@@ -31505,10 +31505,10 @@
         <v>0</v>
       </c>
       <c r="S124" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T124" t="n">
-        <v>6.75</v>
+        <v>6.33</v>
       </c>
       <c r="U124" t="n">
         <v>0</v>
@@ -31762,13 +31762,13 @@
         <v>0</v>
       </c>
       <c r="S127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T127" t="n">
-        <v>6</v>
+        <v>9.75</v>
       </c>
       <c r="U127" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V127" t="n">
         <v>0</v>
@@ -31849,10 +31849,10 @@
         <v>0</v>
       </c>
       <c r="S128" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T128" t="n">
-        <v>5.67</v>
+        <v>5.25</v>
       </c>
       <c r="U128" t="n">
         <v>0</v>
@@ -31934,10 +31934,10 @@
         <v>0</v>
       </c>
       <c r="S129" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T129" t="n">
-        <v>5.33</v>
+        <v>5.5</v>
       </c>
       <c r="U129" t="n">
         <v>0</v>
@@ -32189,10 +32189,10 @@
         <v>0</v>
       </c>
       <c r="S132" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T132" t="n">
-        <v>6</v>
+        <v>6.12</v>
       </c>
       <c r="U132" t="n">
         <v>0</v>
@@ -32426,10 +32426,10 @@
       <c r="Q135" t="inlineStr"/>
       <c r="R135" t="inlineStr"/>
       <c r="S135" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T135" t="n">
-        <v>5.83</v>
+        <v>6.12</v>
       </c>
       <c r="U135" t="n">
         <v>0</v>
@@ -32487,16 +32487,16 @@
       <c r="Q136" t="inlineStr"/>
       <c r="R136" t="inlineStr"/>
       <c r="S136" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T136" t="n">
-        <v>5.5</v>
+        <v>5.88</v>
       </c>
       <c r="U136" t="n">
         <v>0</v>
       </c>
       <c r="V136" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W136" t="inlineStr"/>
       <c r="X136" t="inlineStr"/>
@@ -32792,10 +32792,10 @@
       <c r="Q141" t="inlineStr"/>
       <c r="R141" t="inlineStr"/>
       <c r="S141" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T141" t="n">
-        <v>5.5</v>
+        <v>5.25</v>
       </c>
       <c r="U141" t="n">
         <v>0</v>
@@ -33293,10 +33293,10 @@
         <v>1</v>
       </c>
       <c r="S148" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T148" t="n">
-        <v>6</v>
+        <v>6.12</v>
       </c>
       <c r="U148" t="n">
         <v>0</v>
@@ -33987,10 +33987,10 @@
         <v>0</v>
       </c>
       <c r="S156" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T156" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U156" t="n">
         <v>0</v>
@@ -34248,10 +34248,10 @@
         <v>0</v>
       </c>
       <c r="S159" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T159" t="n">
-        <v>5.67</v>
+        <v>6</v>
       </c>
       <c r="U159" t="n">
         <v>0</v>
@@ -34335,10 +34335,10 @@
         <v>0</v>
       </c>
       <c r="S160" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T160" t="n">
-        <v>6.67</v>
+        <v>6.62</v>
       </c>
       <c r="U160" t="n">
         <v>0</v>
@@ -34509,16 +34509,16 @@
         <v>0</v>
       </c>
       <c r="S162" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T162" t="n">
-        <v>5</v>
+        <v>6.33</v>
       </c>
       <c r="U162" t="n">
         <v>0</v>
       </c>
       <c r="V162" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="W162" t="n">
         <v>2</v>
@@ -34768,10 +34768,10 @@
         <v>0</v>
       </c>
       <c r="S165" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T165" t="n">
-        <v>6.25</v>
+        <v>6.17</v>
       </c>
       <c r="U165" t="n">
         <v>0</v>
@@ -34942,7 +34942,7 @@
         <v>0</v>
       </c>
       <c r="S167" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T167" t="n">
         <v>6</v>
@@ -35029,10 +35029,10 @@
         <v>0</v>
       </c>
       <c r="S168" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T168" t="n">
-        <v>5.83</v>
+        <v>6</v>
       </c>
       <c r="U168" t="n">
         <v>0</v>
@@ -35543,10 +35543,10 @@
         <v>0</v>
       </c>
       <c r="S174" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T174" t="n">
-        <v>5.75</v>
+        <v>5.83</v>
       </c>
       <c r="U174" t="n">
         <v>0</v>
@@ -35713,7 +35713,7 @@
         <v>0</v>
       </c>
       <c r="S176" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T176" t="n">
         <v>6</v>
@@ -36911,10 +36911,10 @@
       <c r="Q194" t="inlineStr"/>
       <c r="R194" t="inlineStr"/>
       <c r="S194" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T194" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U194" t="n">
         <v>0</v>
@@ -37347,10 +37347,10 @@
         <v>1</v>
       </c>
       <c r="S4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T4" t="n">
-        <v>8.5</v>
+        <v>7.75</v>
       </c>
       <c r="U4" t="n">
         <v>2</v>
@@ -37497,10 +37497,10 @@
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T6" t="n">
-        <v>7</v>
+        <v>6.62</v>
       </c>
       <c r="U6" t="n">
         <v>1</v>
@@ -37580,10 +37580,10 @@
         <v>0</v>
       </c>
       <c r="S7" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T7" t="n">
-        <v>6.67</v>
+        <v>6.38</v>
       </c>
       <c r="U7" t="n">
         <v>1</v>
@@ -37754,13 +37754,13 @@
         <v>2</v>
       </c>
       <c r="S9" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T9" t="n">
-        <v>5.83</v>
+        <v>6.88</v>
       </c>
       <c r="U9" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V9" t="n">
         <v>0</v>
@@ -37841,10 +37841,10 @@
         <v>3</v>
       </c>
       <c r="S10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T10" t="n">
-        <v>8.25</v>
+        <v>7.33</v>
       </c>
       <c r="U10" t="n">
         <v>1</v>
@@ -38100,16 +38100,16 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T13" t="n">
-        <v>6.17</v>
+        <v>6.5</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
       </c>
       <c r="V13" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W13" t="n">
         <v>4</v>
@@ -38272,16 +38272,16 @@
         <v>1</v>
       </c>
       <c r="S15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T15" t="n">
-        <v>5.17</v>
+        <v>5.38</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
       </c>
       <c r="V15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W15" t="n">
         <v>0</v>
@@ -38533,10 +38533,10 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T18" t="n">
-        <v>5.83</v>
+        <v>5.62</v>
       </c>
       <c r="U18" t="n">
         <v>0</v>
@@ -38598,10 +38598,10 @@
       <c r="Q19" t="inlineStr"/>
       <c r="R19" t="inlineStr"/>
       <c r="S19" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T19" t="n">
-        <v>6</v>
+        <v>5.75</v>
       </c>
       <c r="U19" t="n">
         <v>0</v>
@@ -38681,13 +38681,13 @@
         <v>1</v>
       </c>
       <c r="S20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T20" t="n">
-        <v>0</v>
+        <v>10.5</v>
       </c>
       <c r="U20" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V20" t="n">
         <v>0</v>
@@ -38855,10 +38855,10 @@
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T22" t="n">
-        <v>5</v>
+        <v>5.25</v>
       </c>
       <c r="U22" t="n">
         <v>0</v>
@@ -39203,10 +39203,10 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T26" t="n">
-        <v>7.75</v>
+        <v>7.17</v>
       </c>
       <c r="U26" t="n">
         <v>1</v>
@@ -39464,10 +39464,10 @@
         <v>2</v>
       </c>
       <c r="S29" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T29" t="n">
-        <v>6.33</v>
+        <v>5.25</v>
       </c>
       <c r="U29" t="n">
         <v>0</v>
@@ -39636,10 +39636,10 @@
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T31" t="n">
-        <v>6.83</v>
+        <v>6.5</v>
       </c>
       <c r="U31" t="n">
         <v>1</v>
@@ -39808,13 +39808,13 @@
         <v>0</v>
       </c>
       <c r="S33" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T33" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U33" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V33" t="n">
         <v>0</v>
@@ -40152,10 +40152,10 @@
         <v>0</v>
       </c>
       <c r="S37" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T37" t="n">
-        <v>10.83</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="U37" t="n">
         <v>4</v>
@@ -40400,10 +40400,10 @@
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr"/>
       <c r="S41" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T41" t="n">
-        <v>7.5</v>
+        <v>6.67</v>
       </c>
       <c r="U41" t="n">
         <v>1</v>
@@ -40461,10 +40461,10 @@
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr"/>
       <c r="S42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T42" t="n">
-        <v>10</v>
+        <v>8.67</v>
       </c>
       <c r="U42" t="n">
         <v>2</v>
@@ -40890,13 +40890,13 @@
         <v>0</v>
       </c>
       <c r="S47" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T47" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V47" t="n">
         <v>0</v>
@@ -40977,10 +40977,10 @@
         <v>0</v>
       </c>
       <c r="S48" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T48" t="n">
-        <v>5.5</v>
+        <v>5.62</v>
       </c>
       <c r="U48" t="n">
         <v>0</v>
@@ -41149,10 +41149,10 @@
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T50" t="n">
-        <v>6</v>
+        <v>5.83</v>
       </c>
       <c r="U50" t="n">
         <v>0</v>
@@ -41323,13 +41323,13 @@
         <v>0</v>
       </c>
       <c r="S52" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T52" t="n">
-        <v>7.17</v>
+        <v>7.88</v>
       </c>
       <c r="U52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V52" t="n">
         <v>0</v>
@@ -41408,10 +41408,10 @@
         <v>1</v>
       </c>
       <c r="S53" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T53" t="n">
-        <v>5.33</v>
+        <v>5.5</v>
       </c>
       <c r="U53" t="n">
         <v>0</v>
@@ -41495,7 +41495,7 @@
         <v>0</v>
       </c>
       <c r="S54" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T54" t="n">
         <v>6</v>
@@ -41580,13 +41580,13 @@
         <v>0</v>
       </c>
       <c r="S55" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T55" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="U55" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V55" t="n">
         <v>0</v>
@@ -41665,10 +41665,10 @@
         <v>0</v>
       </c>
       <c r="S56" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T56" t="n">
-        <v>5.75</v>
+        <v>5.83</v>
       </c>
       <c r="U56" t="n">
         <v>0</v>
@@ -41839,10 +41839,10 @@
         <v>0</v>
       </c>
       <c r="S58" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T58" t="n">
-        <v>5.83</v>
+        <v>5.75</v>
       </c>
       <c r="U58" t="n">
         <v>0</v>
@@ -42011,10 +42011,10 @@
         <v>0</v>
       </c>
       <c r="S60" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T60" t="n">
-        <v>6</v>
+        <v>6.25</v>
       </c>
       <c r="U60" t="n">
         <v>0</v>
@@ -42096,13 +42096,13 @@
         <v>0</v>
       </c>
       <c r="S61" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T61" t="n">
-        <v>8.17</v>
+        <v>8.619999999999999</v>
       </c>
       <c r="U61" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V61" t="n">
         <v>1</v>
@@ -42222,10 +42222,10 @@
       <c r="Q63" t="inlineStr"/>
       <c r="R63" t="inlineStr"/>
       <c r="S63" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T63" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U63" t="n">
         <v>0</v>
@@ -42405,10 +42405,10 @@
       <c r="Q66" t="inlineStr"/>
       <c r="R66" t="inlineStr"/>
       <c r="S66" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T66" t="n">
-        <v>10</v>
+        <v>8.25</v>
       </c>
       <c r="U66" t="n">
         <v>1</v>
@@ -42466,13 +42466,13 @@
       <c r="Q67" t="inlineStr"/>
       <c r="R67" t="inlineStr"/>
       <c r="S67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T67" t="n">
-        <v>0</v>
+        <v>9.5</v>
       </c>
       <c r="U67" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V67" t="n">
         <v>0</v>
@@ -43420,10 +43420,10 @@
       <c r="Q79" t="inlineStr"/>
       <c r="R79" t="inlineStr"/>
       <c r="S79" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T79" t="n">
-        <v>5.5</v>
+        <v>5.67</v>
       </c>
       <c r="U79" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore: aggiornamento automatico dati fantacalcio 2026-10-04
</commit_message>
<xml_diff>
--- a/export/lista_asta.xlsx
+++ b/export/lista_asta.xlsx
@@ -14,7 +14,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Portieri'!$A$1:$AA$65</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Difensori'!$A$1:$AA$191</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Difensori'!$A$1:$AA$192</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Centrocampisti'!$A$1:$AA$195</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Attaccanti'!$A$1:$AA$88</definedName>
   </definedNames>
@@ -5698,7 +5698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AA191"/>
+  <dimension ref="A1:AA192"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -17428,73 +17428,51 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Dodò</t>
+          <t>Mitaj</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>Dd;E</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>Fiorentina</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E144" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="F144" t="n">
-        <v>2</v>
-      </c>
-      <c r="G144" s="6" t="inlineStr">
-        <is>
-          <t>Low Cost</t>
-        </is>
-      </c>
-      <c r="H144" t="n">
-        <v>68.3</v>
-      </c>
-      <c r="I144" t="inlineStr">
-        <is>
-          <t>Affare</t>
-        </is>
-      </c>
-      <c r="J144" t="n">
-        <v>36</v>
-      </c>
-      <c r="K144" t="n">
-        <v>5.99</v>
-      </c>
-      <c r="L144" t="n">
-        <v>6.03</v>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="G144" s="5" t="inlineStr">
+        <is>
+          <t>3a Fascia</t>
+        </is>
+      </c>
+      <c r="H144" t="inlineStr"/>
+      <c r="I144" t="inlineStr"/>
+      <c r="J144" t="inlineStr"/>
+      <c r="K144" t="inlineStr"/>
+      <c r="L144" t="inlineStr"/>
       <c r="M144" t="n">
-        <v>3</v>
-      </c>
-      <c r="N144" t="n">
-        <v>-0.01</v>
-      </c>
-      <c r="O144" t="n">
-        <v>0.675</v>
-      </c>
-      <c r="P144" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q144" t="n">
-        <v>2</v>
-      </c>
-      <c r="R144" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="N144" t="inlineStr"/>
+      <c r="O144" t="inlineStr"/>
+      <c r="P144" t="inlineStr"/>
+      <c r="Q144" t="inlineStr"/>
+      <c r="R144" t="inlineStr"/>
       <c r="S144" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T144" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U144" t="n">
         <v>0</v>
@@ -17502,12 +17480,8 @@
       <c r="V144" t="n">
         <v>0</v>
       </c>
-      <c r="W144" t="n">
-        <v>7</v>
-      </c>
-      <c r="X144" t="n">
-        <v>0</v>
-      </c>
+      <c r="W144" t="inlineStr"/>
+      <c r="X144" t="inlineStr"/>
       <c r="Y144" t="inlineStr"/>
       <c r="Z144" t="inlineStr"/>
       <c r="AA144" t="inlineStr"/>
@@ -17515,24 +17489,24 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Cabal</t>
+          <t>Dodò</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>B;Ds;E</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Fiorentina</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E145" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F145" t="n">
         <v>2</v>
@@ -17543,7 +17517,7 @@
         </is>
       </c>
       <c r="H145" t="n">
-        <v>65.2</v>
+        <v>68.3</v>
       </c>
       <c r="I145" t="inlineStr">
         <is>
@@ -17551,37 +17525,37 @@
         </is>
       </c>
       <c r="J145" t="n">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="K145" t="n">
-        <v>5.94</v>
+        <v>5.99</v>
       </c>
       <c r="L145" t="n">
-        <v>6.56</v>
+        <v>6.03</v>
       </c>
       <c r="M145" t="n">
         <v>3</v>
       </c>
       <c r="N145" t="n">
-        <v>0.53</v>
+        <v>-0.01</v>
       </c>
       <c r="O145" t="n">
-        <v>0.298</v>
+        <v>0.675</v>
       </c>
       <c r="P145" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q145" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="R145" t="n">
         <v>0</v>
       </c>
       <c r="S145" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T145" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="U145" t="n">
         <v>0</v>
@@ -17590,7 +17564,7 @@
         <v>0</v>
       </c>
       <c r="W145" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="X145" t="n">
         <v>0</v>
@@ -17602,24 +17576,24 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Idrissi R.</t>
+          <t>Cabal</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>Ds;E</t>
+          <t>B;Ds;E</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E146" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F146" t="n">
         <v>2</v>
@@ -17630,7 +17604,7 @@
         </is>
       </c>
       <c r="H146" t="n">
-        <v>62</v>
+        <v>65.2</v>
       </c>
       <c r="I146" t="inlineStr">
         <is>
@@ -17638,20 +17612,22 @@
         </is>
       </c>
       <c r="J146" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="K146" t="n">
-        <v>5.82</v>
+        <v>5.94</v>
       </c>
       <c r="L146" t="n">
-        <v>6.09</v>
+        <v>6.56</v>
       </c>
       <c r="M146" t="n">
-        <v>1</v>
-      </c>
-      <c r="N146" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="N146" t="n">
+        <v>0.53</v>
+      </c>
       <c r="O146" t="n">
-        <v>0.447</v>
+        <v>0.298</v>
       </c>
       <c r="P146" t="n">
         <v>2</v>
@@ -17675,7 +17651,7 @@
         <v>0</v>
       </c>
       <c r="W146" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="X146" t="n">
         <v>0</v>
@@ -17687,17 +17663,17 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>De Silvestri</t>
+          <t>Idrissi R.</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>Dd;E</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>Bologna</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="D147" t="n">
@@ -17715,7 +17691,7 @@
         </is>
       </c>
       <c r="H147" t="n">
-        <v>49.9</v>
+        <v>62</v>
       </c>
       <c r="I147" t="inlineStr">
         <is>
@@ -17723,25 +17699,23 @@
         </is>
       </c>
       <c r="J147" t="n">
-        <v>10</v>
+        <v>17</v>
       </c>
       <c r="K147" t="n">
-        <v>6.05</v>
+        <v>5.82</v>
       </c>
       <c r="L147" t="n">
-        <v>5.95</v>
+        <v>6.09</v>
       </c>
       <c r="M147" t="n">
-        <v>3</v>
-      </c>
-      <c r="N147" t="n">
-        <v>-0.34</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N147" t="inlineStr"/>
       <c r="O147" t="n">
-        <v>0.333</v>
+        <v>0.447</v>
       </c>
       <c r="P147" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q147" t="n">
         <v>0</v>
@@ -17750,10 +17724,10 @@
         <v>0</v>
       </c>
       <c r="S147" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T147" t="n">
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="U147" t="n">
         <v>0</v>
@@ -17762,7 +17736,7 @@
         <v>0</v>
       </c>
       <c r="W147" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X147" t="n">
         <v>0</v>
@@ -17774,24 +17748,24 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Pellegrini Lu.</t>
+          <t>De Silvestri</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>Ds;E</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Bologna</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E148" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F148" t="n">
         <v>2</v>
@@ -17802,7 +17776,7 @@
         </is>
       </c>
       <c r="H148" t="n">
-        <v>47.5</v>
+        <v>49.9</v>
       </c>
       <c r="I148" t="inlineStr">
         <is>
@@ -17810,25 +17784,25 @@
         </is>
       </c>
       <c r="J148" t="n">
-        <v>24</v>
+        <v>10</v>
       </c>
       <c r="K148" t="n">
-        <v>5.85</v>
+        <v>6.05</v>
       </c>
       <c r="L148" t="n">
-        <v>5.81</v>
+        <v>5.95</v>
       </c>
       <c r="M148" t="n">
         <v>3</v>
       </c>
       <c r="N148" t="n">
-        <v>-0.17</v>
+        <v>-0.34</v>
       </c>
       <c r="O148" t="n">
-        <v>0.526</v>
+        <v>0.333</v>
       </c>
       <c r="P148" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q148" t="n">
         <v>0</v>
@@ -17837,10 +17811,10 @@
         <v>0</v>
       </c>
       <c r="S148" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T148" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="U148" t="n">
         <v>0</v>
@@ -17849,7 +17823,7 @@
         <v>0</v>
       </c>
       <c r="W148" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="X148" t="n">
         <v>0</v>
@@ -17861,27 +17835,27 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Van Der Brempt</t>
+          <t>Pellegrini Lu.</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Dd;E</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="D149" t="n">
         <v>1</v>
       </c>
       <c r="E149" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F149" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G149" s="6" t="inlineStr">
         <is>
@@ -17889,7 +17863,7 @@
         </is>
       </c>
       <c r="H149" t="n">
-        <v>43.2</v>
+        <v>47.5</v>
       </c>
       <c r="I149" t="inlineStr">
         <is>
@@ -17897,28 +17871,28 @@
         </is>
       </c>
       <c r="J149" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="K149" t="n">
-        <v>5.96</v>
+        <v>5.85</v>
       </c>
       <c r="L149" t="n">
-        <v>5.96</v>
+        <v>5.81</v>
       </c>
       <c r="M149" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N149" t="n">
-        <v>0.04</v>
+        <v>-0.17</v>
       </c>
       <c r="O149" t="n">
-        <v>0.421</v>
+        <v>0.526</v>
       </c>
       <c r="P149" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q149" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R149" t="n">
         <v>0</v>
@@ -17936,7 +17910,7 @@
         <v>0</v>
       </c>
       <c r="W149" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="X149" t="n">
         <v>0</v>
@@ -17948,27 +17922,27 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Sverko</t>
+          <t>Van Der Brempt</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>Ds;Dc</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E150" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F150" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G150" s="6" t="inlineStr">
         <is>
@@ -17976,7 +17950,7 @@
         </is>
       </c>
       <c r="H150" t="n">
-        <v>42.8</v>
+        <v>43.2</v>
       </c>
       <c r="I150" t="inlineStr">
         <is>
@@ -17987,23 +17961,25 @@
         <v>14</v>
       </c>
       <c r="K150" t="n">
-        <v>5.75</v>
+        <v>5.96</v>
       </c>
       <c r="L150" t="n">
-        <v>5.86</v>
+        <v>5.96</v>
       </c>
       <c r="M150" t="n">
-        <v>1</v>
-      </c>
-      <c r="N150" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="N150" t="n">
+        <v>0.04</v>
+      </c>
       <c r="O150" t="n">
-        <v>0.368</v>
+        <v>0.421</v>
       </c>
       <c r="P150" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q150" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R150" t="n">
         <v>0</v>
@@ -18021,7 +17997,7 @@
         <v>0</v>
       </c>
       <c r="W150" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X150" t="n">
         <v>0</v>
@@ -18033,35 +18009,35 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Terracciano F.</t>
+          <t>Sverko</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>B;Dd;Ds</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>Milan</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E151" t="n">
+        <v>7</v>
+      </c>
+      <c r="F151" t="n">
         <v>4</v>
       </c>
-      <c r="F151" t="n">
-        <v>2</v>
-      </c>
       <c r="G151" s="6" t="inlineStr">
         <is>
           <t>Low Cost</t>
         </is>
       </c>
       <c r="H151" t="n">
-        <v>42.6</v>
+        <v>42.8</v>
       </c>
       <c r="I151" t="inlineStr">
         <is>
@@ -18069,25 +18045,23 @@
         </is>
       </c>
       <c r="J151" t="n">
-        <v>35</v>
+        <v>14</v>
       </c>
       <c r="K151" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="L151" t="n">
         <v>5.86</v>
       </c>
-      <c r="L151" t="n">
-        <v>5.83</v>
-      </c>
       <c r="M151" t="n">
-        <v>3</v>
-      </c>
-      <c r="N151" t="n">
-        <v>0.14</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N151" t="inlineStr"/>
       <c r="O151" t="n">
-        <v>0.535</v>
+        <v>0.368</v>
       </c>
       <c r="P151" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="Q151" t="n">
         <v>0</v>
@@ -18108,7 +18082,7 @@
         <v>0</v>
       </c>
       <c r="W151" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="X151" t="n">
         <v>0</v>
@@ -18120,24 +18094,24 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Biraghi</t>
+          <t>Terracciano F.</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>B;Ds;E</t>
+          <t>B;Dd;Ds</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>Torino</t>
+          <t>Milan</t>
         </is>
       </c>
       <c r="D152" t="n">
         <v>1</v>
       </c>
       <c r="E152" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F152" t="n">
         <v>2</v>
@@ -18148,7 +18122,7 @@
         </is>
       </c>
       <c r="H152" t="n">
-        <v>35.2</v>
+        <v>42.6</v>
       </c>
       <c r="I152" t="inlineStr">
         <is>
@@ -18156,25 +18130,25 @@
         </is>
       </c>
       <c r="J152" t="n">
-        <v>11</v>
+        <v>35</v>
       </c>
       <c r="K152" t="n">
-        <v>5.59</v>
+        <v>5.86</v>
       </c>
       <c r="L152" t="n">
-        <v>5.59</v>
+        <v>5.83</v>
       </c>
       <c r="M152" t="n">
         <v>3</v>
       </c>
       <c r="N152" t="n">
-        <v>-0.36</v>
+        <v>0.14</v>
       </c>
       <c r="O152" t="n">
-        <v>0.526</v>
+        <v>0.535</v>
       </c>
       <c r="P152" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Q152" t="n">
         <v>0</v>
@@ -18195,7 +18169,7 @@
         <v>0</v>
       </c>
       <c r="W152" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="X152" t="n">
         <v>0</v>
@@ -18207,17 +18181,17 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Lazzari</t>
+          <t>Biraghi</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Dd;E</t>
+          <t>B;Ds;E</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>Lazio</t>
+          <t>Torino</t>
         </is>
       </c>
       <c r="D153" t="n">
@@ -18235,7 +18209,7 @@
         </is>
       </c>
       <c r="H153" t="n">
-        <v>32</v>
+        <v>35.2</v>
       </c>
       <c r="I153" t="inlineStr">
         <is>
@@ -18243,22 +18217,22 @@
         </is>
       </c>
       <c r="J153" t="n">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="K153" t="n">
-        <v>5.79</v>
+        <v>5.59</v>
       </c>
       <c r="L153" t="n">
-        <v>5.74</v>
+        <v>5.59</v>
       </c>
       <c r="M153" t="n">
         <v>3</v>
       </c>
       <c r="N153" t="n">
-        <v>-0.13</v>
+        <v>-0.36</v>
       </c>
       <c r="O153" t="n">
-        <v>0.553</v>
+        <v>0.526</v>
       </c>
       <c r="P153" t="n">
         <v>0</v>
@@ -18282,7 +18256,7 @@
         <v>0</v>
       </c>
       <c r="W153" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="X153" t="n">
         <v>0</v>
@@ -18294,21 +18268,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Sabelli</t>
+          <t>Lazzari</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Dd;Ds;E</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Lazio</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E154" t="n">
         <v>5</v>
@@ -18322,30 +18296,30 @@
         </is>
       </c>
       <c r="H154" t="n">
-        <v>28.2</v>
+        <v>32</v>
       </c>
       <c r="I154" t="inlineStr">
         <is>
-          <t>Equo</t>
+          <t>Affare</t>
         </is>
       </c>
       <c r="J154" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="K154" t="n">
-        <v>5.81</v>
+        <v>5.79</v>
       </c>
       <c r="L154" t="n">
-        <v>5.65</v>
+        <v>5.74</v>
       </c>
       <c r="M154" t="n">
         <v>3</v>
       </c>
       <c r="N154" t="n">
-        <v>-0.24</v>
+        <v>-0.13</v>
       </c>
       <c r="O154" t="n">
-        <v>0.649</v>
+        <v>0.553</v>
       </c>
       <c r="P154" t="n">
         <v>0</v>
@@ -18357,10 +18331,10 @@
         <v>0</v>
       </c>
       <c r="S154" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T154" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U154" t="n">
         <v>0</v>
@@ -18369,7 +18343,7 @@
         <v>0</v>
       </c>
       <c r="W154" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X154" t="n">
         <v>0</v>
@@ -18381,21 +18355,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Ebosse</t>
+          <t>Sabelli</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Ds;Dc</t>
+          <t>Dd;Ds;E</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>Udinese</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E155" t="n">
         <v>5</v>
@@ -18409,7 +18383,7 @@
         </is>
       </c>
       <c r="H155" t="n">
-        <v>28.1</v>
+        <v>28.2</v>
       </c>
       <c r="I155" t="inlineStr">
         <is>
@@ -18417,38 +18391,38 @@
         </is>
       </c>
       <c r="J155" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="K155" t="n">
-        <v>5.75</v>
+        <v>5.81</v>
       </c>
       <c r="L155" t="n">
-        <v>5.72</v>
+        <v>5.65</v>
       </c>
       <c r="M155" t="n">
         <v>3</v>
       </c>
       <c r="N155" t="n">
-        <v>2.44</v>
+        <v>-0.24</v>
       </c>
       <c r="O155" t="n">
-        <v>0.158</v>
+        <v>0.649</v>
       </c>
       <c r="P155" t="n">
         <v>0</v>
       </c>
       <c r="Q155" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R155" t="n">
         <v>0</v>
       </c>
       <c r="S155" t="n">
+        <v>1</v>
+      </c>
+      <c r="T155" t="n">
         <v>5</v>
       </c>
-      <c r="T155" t="n">
-        <v>5.6</v>
-      </c>
       <c r="U155" t="n">
         <v>0</v>
       </c>
@@ -18456,7 +18430,7 @@
         <v>0</v>
       </c>
       <c r="W155" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="X155" t="n">
         <v>0</v>
@@ -18468,24 +18442,24 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Marianucci</t>
+          <t>Ebosse</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Dc</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>Napoli</t>
+          <t>Udinese</t>
         </is>
       </c>
       <c r="D156" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E156" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F156" t="n">
         <v>2</v>
@@ -18496,30 +18470,30 @@
         </is>
       </c>
       <c r="H156" t="n">
-        <v>25.8</v>
+        <v>28.1</v>
       </c>
       <c r="I156" t="inlineStr">
         <is>
-          <t>Affare</t>
+          <t>Equo</t>
         </is>
       </c>
       <c r="J156" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="K156" t="n">
-        <v>5.73</v>
+        <v>5.75</v>
       </c>
       <c r="L156" t="n">
-        <v>5.73</v>
+        <v>5.72</v>
       </c>
       <c r="M156" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N156" t="n">
-        <v>0</v>
+        <v>2.44</v>
       </c>
       <c r="O156" t="n">
-        <v>0.316</v>
+        <v>0.158</v>
       </c>
       <c r="P156" t="n">
         <v>0</v>
@@ -18531,10 +18505,10 @@
         <v>0</v>
       </c>
       <c r="S156" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="T156" t="n">
-        <v>0</v>
+        <v>5.6</v>
       </c>
       <c r="U156" t="n">
         <v>0</v>
@@ -18543,7 +18517,7 @@
         <v>0</v>
       </c>
       <c r="W156" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="X156" t="n">
         <v>0</v>
@@ -18555,7 +18529,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Rugani</t>
+          <t>Marianucci</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
@@ -18565,7 +18539,7 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>Juventus</t>
+          <t>Napoli</t>
         </is>
       </c>
       <c r="D157" t="n">
@@ -18583,7 +18557,7 @@
         </is>
       </c>
       <c r="H157" t="n">
-        <v>25.4</v>
+        <v>25.8</v>
       </c>
       <c r="I157" t="inlineStr">
         <is>
@@ -18591,28 +18565,28 @@
         </is>
       </c>
       <c r="J157" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="K157" t="n">
-        <v>5.69</v>
+        <v>5.73</v>
       </c>
       <c r="L157" t="n">
-        <v>5.56</v>
+        <v>5.73</v>
       </c>
       <c r="M157" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N157" t="n">
-        <v>3.14</v>
+        <v>0</v>
       </c>
       <c r="O157" t="n">
-        <v>0.193</v>
+        <v>0.316</v>
       </c>
       <c r="P157" t="n">
         <v>0</v>
       </c>
       <c r="Q157" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R157" t="n">
         <v>0</v>
@@ -18642,7 +18616,7 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>Ziolkowski</t>
+          <t>Rugani</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
@@ -18652,17 +18626,17 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Juventus</t>
         </is>
       </c>
       <c r="D158" t="n">
         <v>1</v>
       </c>
       <c r="E158" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F158" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G158" s="6" t="inlineStr">
         <is>
@@ -18670,28 +18644,30 @@
         </is>
       </c>
       <c r="H158" t="n">
-        <v>21.4</v>
+        <v>25.4</v>
       </c>
       <c r="I158" t="inlineStr">
         <is>
-          <t>Equo</t>
+          <t>Affare</t>
         </is>
       </c>
       <c r="J158" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="K158" t="n">
-        <v>5.94</v>
+        <v>5.69</v>
       </c>
       <c r="L158" t="n">
-        <v>5.78</v>
+        <v>5.56</v>
       </c>
       <c r="M158" t="n">
-        <v>1</v>
-      </c>
-      <c r="N158" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="N158" t="n">
+        <v>3.14</v>
+      </c>
       <c r="O158" t="n">
-        <v>0.237</v>
+        <v>0.193</v>
       </c>
       <c r="P158" t="n">
         <v>0</v>
@@ -18715,7 +18691,7 @@
         <v>0</v>
       </c>
       <c r="W158" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X158" t="n">
         <v>0</v>
@@ -18727,35 +18703,35 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Candè</t>
+          <t>Ziolkowski</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Ds;Dc</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E159" t="n">
+        <v>7</v>
+      </c>
+      <c r="F159" t="n">
         <v>4</v>
       </c>
-      <c r="F159" t="n">
-        <v>2</v>
-      </c>
       <c r="G159" s="6" t="inlineStr">
         <is>
           <t>Low Cost</t>
         </is>
       </c>
       <c r="H159" t="n">
-        <v>18.9</v>
+        <v>21.4</v>
       </c>
       <c r="I159" t="inlineStr">
         <is>
@@ -18763,22 +18739,20 @@
         </is>
       </c>
       <c r="J159" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="K159" t="n">
-        <v>5.69</v>
+        <v>5.94</v>
       </c>
       <c r="L159" t="n">
-        <v>5.56</v>
+        <v>5.78</v>
       </c>
       <c r="M159" t="n">
-        <v>2</v>
-      </c>
-      <c r="N159" t="n">
-        <v>-0.26</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="N159" t="inlineStr"/>
       <c r="O159" t="n">
-        <v>0.329</v>
+        <v>0.237</v>
       </c>
       <c r="P159" t="n">
         <v>0</v>
@@ -18802,7 +18776,7 @@
         <v>0</v>
       </c>
       <c r="W159" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X159" t="n">
         <v>0</v>
@@ -18814,17 +18788,17 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Casale</t>
+          <t>Candè</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Dc</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>Bologna</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="D160" t="n">
@@ -18842,7 +18816,7 @@
         </is>
       </c>
       <c r="H160" t="n">
-        <v>18.4</v>
+        <v>18.9</v>
       </c>
       <c r="I160" t="inlineStr">
         <is>
@@ -18850,22 +18824,22 @@
         </is>
       </c>
       <c r="J160" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="K160" t="n">
-        <v>5.65</v>
+        <v>5.69</v>
       </c>
       <c r="L160" t="n">
-        <v>5.65</v>
+        <v>5.56</v>
       </c>
       <c r="M160" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N160" t="n">
-        <v>0.11</v>
+        <v>-0.26</v>
       </c>
       <c r="O160" t="n">
-        <v>0.386</v>
+        <v>0.329</v>
       </c>
       <c r="P160" t="n">
         <v>0</v>
@@ -18889,7 +18863,7 @@
         <v>0</v>
       </c>
       <c r="W160" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X160" t="n">
         <v>0</v>
@@ -18901,7 +18875,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>Jean</t>
+          <t>Casale</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
@@ -18911,11 +18885,11 @@
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Bologna</t>
         </is>
       </c>
       <c r="D161" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E161" t="n">
         <v>4</v>
@@ -18929,7 +18903,7 @@
         </is>
       </c>
       <c r="H161" t="n">
-        <v>18.2</v>
+        <v>18.4</v>
       </c>
       <c r="I161" t="inlineStr">
         <is>
@@ -18937,22 +18911,22 @@
         </is>
       </c>
       <c r="J161" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="K161" t="n">
-        <v>5.8</v>
+        <v>5.65</v>
       </c>
       <c r="L161" t="n">
-        <v>5.7</v>
+        <v>5.65</v>
       </c>
       <c r="M161" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N161" t="n">
-        <v>-0.05</v>
+        <v>0.11</v>
       </c>
       <c r="O161" t="n">
-        <v>0.303</v>
+        <v>0.386</v>
       </c>
       <c r="P161" t="n">
         <v>0</v>
@@ -18976,7 +18950,7 @@
         <v>0</v>
       </c>
       <c r="W161" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X161" t="n">
         <v>0</v>
@@ -18988,58 +18962,58 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Goglichidze</t>
+          <t>Jean</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Dd;Dc</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="D162" t="n">
         <v>1</v>
       </c>
       <c r="E162" t="n">
+        <v>4</v>
+      </c>
+      <c r="F162" t="n">
+        <v>2</v>
+      </c>
+      <c r="G162" s="6" t="inlineStr">
+        <is>
+          <t>Low Cost</t>
+        </is>
+      </c>
+      <c r="H162" t="n">
+        <v>18.2</v>
+      </c>
+      <c r="I162" t="inlineStr">
+        <is>
+          <t>Equo</t>
+        </is>
+      </c>
+      <c r="J162" t="n">
         <v>5</v>
       </c>
-      <c r="F162" t="n">
-        <v>2</v>
-      </c>
-      <c r="G162" s="6" t="inlineStr">
-        <is>
-          <t>Low Cost</t>
-        </is>
-      </c>
-      <c r="H162" t="n">
-        <v>17.4</v>
-      </c>
-      <c r="I162" t="inlineStr">
-        <is>
-          <t>Equo</t>
-        </is>
-      </c>
-      <c r="J162" t="n">
-        <v>6</v>
-      </c>
       <c r="K162" t="n">
-        <v>5.75</v>
+        <v>5.8</v>
       </c>
       <c r="L162" t="n">
-        <v>5.58</v>
+        <v>5.7</v>
       </c>
       <c r="M162" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N162" t="n">
-        <v>2.01</v>
+        <v>-0.05</v>
       </c>
       <c r="O162" t="n">
-        <v>0.342</v>
+        <v>0.303</v>
       </c>
       <c r="P162" t="n">
         <v>0</v>
@@ -19063,7 +19037,7 @@
         <v>0</v>
       </c>
       <c r="W162" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="X162" t="n">
         <v>0</v>
@@ -19075,56 +19049,58 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>Moreno M.</t>
+          <t>Goglichidze</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Dc</t>
+          <t>Dd;Dc</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="D163" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E163" t="n">
+        <v>5</v>
+      </c>
+      <c r="F163" t="n">
+        <v>2</v>
+      </c>
+      <c r="G163" s="6" t="inlineStr">
+        <is>
+          <t>Low Cost</t>
+        </is>
+      </c>
+      <c r="H163" t="n">
+        <v>17.4</v>
+      </c>
+      <c r="I163" t="inlineStr">
+        <is>
+          <t>Equo</t>
+        </is>
+      </c>
+      <c r="J163" t="n">
         <v>6</v>
       </c>
-      <c r="F163" t="n">
-        <v>3</v>
-      </c>
-      <c r="G163" s="6" t="inlineStr">
-        <is>
-          <t>Low Cost</t>
-        </is>
-      </c>
-      <c r="H163" t="n">
-        <v>16.6</v>
-      </c>
-      <c r="I163" t="inlineStr">
-        <is>
-          <t>Equo</t>
-        </is>
-      </c>
-      <c r="J163" t="n">
-        <v>3</v>
-      </c>
       <c r="K163" t="n">
-        <v>5.67</v>
+        <v>5.75</v>
       </c>
       <c r="L163" t="n">
-        <v>5.67</v>
+        <v>5.58</v>
       </c>
       <c r="M163" t="n">
-        <v>1</v>
-      </c>
-      <c r="N163" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="N163" t="n">
+        <v>2.01</v>
+      </c>
       <c r="O163" t="n">
-        <v>0.079</v>
+        <v>0.342</v>
       </c>
       <c r="P163" t="n">
         <v>0</v>
@@ -19136,10 +19112,10 @@
         <v>0</v>
       </c>
       <c r="S163" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T163" t="n">
-        <v>5.17</v>
+        <v>0</v>
       </c>
       <c r="U163" t="n">
         <v>0</v>
@@ -19148,7 +19124,7 @@
         <v>0</v>
       </c>
       <c r="W163" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="X163" t="n">
         <v>0</v>
@@ -19160,27 +19136,27 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Ndaba</t>
+          <t>Moreno M.</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Ds;E</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E164" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F164" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G164" s="6" t="inlineStr">
         <is>
@@ -19188,7 +19164,7 @@
         </is>
       </c>
       <c r="H164" t="n">
-        <v>15.8</v>
+        <v>16.6</v>
       </c>
       <c r="I164" t="inlineStr">
         <is>
@@ -19196,20 +19172,20 @@
         </is>
       </c>
       <c r="J164" t="n">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="K164" t="n">
-        <v>5.5</v>
+        <v>5.67</v>
       </c>
       <c r="L164" t="n">
-        <v>5.5</v>
+        <v>5.67</v>
       </c>
       <c r="M164" t="n">
         <v>1</v>
       </c>
       <c r="N164" t="inlineStr"/>
       <c r="O164" t="n">
-        <v>0.237</v>
+        <v>0.079</v>
       </c>
       <c r="P164" t="n">
         <v>0</v>
@@ -19221,10 +19197,10 @@
         <v>0</v>
       </c>
       <c r="S164" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T164" t="n">
-        <v>5.5</v>
+        <v>5.17</v>
       </c>
       <c r="U164" t="n">
         <v>0</v>
@@ -19245,27 +19221,27 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Odenthal</t>
+          <t>Ndaba</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Dc</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>Sassuolo</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E165" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F165" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G165" s="6" t="inlineStr">
         <is>
@@ -19273,7 +19249,7 @@
         </is>
       </c>
       <c r="H165" t="n">
-        <v>11</v>
+        <v>15.8</v>
       </c>
       <c r="I165" t="inlineStr">
         <is>
@@ -19281,20 +19257,20 @@
         </is>
       </c>
       <c r="J165" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="K165" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="L165" t="n">
-        <v>0</v>
+        <v>5.5</v>
       </c>
       <c r="M165" t="n">
         <v>1</v>
       </c>
       <c r="N165" t="inlineStr"/>
       <c r="O165" t="n">
-        <v>0</v>
+        <v>0.237</v>
       </c>
       <c r="P165" t="n">
         <v>0</v>
@@ -19306,13 +19282,13 @@
         <v>0</v>
       </c>
       <c r="S165" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T165" t="n">
-        <v>10</v>
+        <v>5.5</v>
       </c>
       <c r="U165" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V165" t="n">
         <v>0</v>
@@ -19330,27 +19306,27 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Otoa</t>
+          <t>Carboni F.</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Dc</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Parma</t>
         </is>
       </c>
       <c r="D166" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E166" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F166" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G166" s="6" t="inlineStr">
         <is>
@@ -19358,7 +19334,7 @@
         </is>
       </c>
       <c r="H166" t="n">
-        <v>11</v>
+        <v>14.2</v>
       </c>
       <c r="I166" t="inlineStr">
         <is>
@@ -19366,22 +19342,22 @@
         </is>
       </c>
       <c r="J166" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="K166" t="n">
-        <v>5.6</v>
+        <v>6</v>
       </c>
       <c r="L166" t="n">
-        <v>5.35</v>
+        <v>6</v>
       </c>
       <c r="M166" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="N166" t="n">
-        <v>0.68</v>
+        <v>2.44</v>
       </c>
       <c r="O166" t="n">
-        <v>0.171</v>
+        <v>0.061</v>
       </c>
       <c r="P166" t="n">
         <v>0</v>
@@ -19393,10 +19369,10 @@
         <v>0</v>
       </c>
       <c r="S166" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T166" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="U166" t="n">
         <v>0</v>
@@ -19405,7 +19381,7 @@
         <v>0</v>
       </c>
       <c r="W166" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X166" t="n">
         <v>0</v>
@@ -19417,27 +19393,27 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Sagrado</t>
+          <t>Odenthal</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Dd;E</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Sassuolo</t>
         </is>
       </c>
       <c r="D167" t="n">
         <v>3</v>
       </c>
       <c r="E167" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F167" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G167" s="6" t="inlineStr">
         <is>
@@ -19445,7 +19421,7 @@
         </is>
       </c>
       <c r="H167" t="n">
-        <v>9.199999999999999</v>
+        <v>11</v>
       </c>
       <c r="I167" t="inlineStr">
         <is>
@@ -19453,20 +19429,20 @@
         </is>
       </c>
       <c r="J167" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="K167" t="n">
-        <v>5.5</v>
+        <v>0</v>
       </c>
       <c r="L167" t="n">
-        <v>5.33</v>
+        <v>0</v>
       </c>
       <c r="M167" t="n">
         <v>1</v>
       </c>
       <c r="N167" t="inlineStr"/>
       <c r="O167" t="n">
-        <v>0.079</v>
+        <v>0</v>
       </c>
       <c r="P167" t="n">
         <v>0</v>
@@ -19478,10 +19454,10 @@
         <v>0</v>
       </c>
       <c r="S167" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T167" t="n">
-        <v>7.5</v>
+        <v>10</v>
       </c>
       <c r="U167" t="n">
         <v>1</v>
@@ -19490,7 +19466,7 @@
         <v>0</v>
       </c>
       <c r="W167" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X167" t="n">
         <v>0</v>
@@ -19502,7 +19478,7 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Kofler</t>
+          <t>Otoa</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
@@ -19512,50 +19488,76 @@
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="D168" t="n">
+        <v>2</v>
+      </c>
+      <c r="E168" t="n">
+        <v>7</v>
+      </c>
+      <c r="F168" t="n">
+        <v>4</v>
+      </c>
+      <c r="G168" s="6" t="inlineStr">
+        <is>
+          <t>Low Cost</t>
+        </is>
+      </c>
+      <c r="H168" t="n">
+        <v>11</v>
+      </c>
+      <c r="I168" t="inlineStr">
+        <is>
+          <t>Equo</t>
+        </is>
+      </c>
+      <c r="J168" t="n">
+        <v>10</v>
+      </c>
+      <c r="K168" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="L168" t="n">
+        <v>5.35</v>
+      </c>
+      <c r="M168" t="n">
+        <v>2</v>
+      </c>
+      <c r="N168" t="n">
+        <v>0.68</v>
+      </c>
+      <c r="O168" t="n">
+        <v>0.171</v>
+      </c>
+      <c r="P168" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q168" t="n">
+        <v>0</v>
+      </c>
+      <c r="R168" t="n">
+        <v>0</v>
+      </c>
+      <c r="S168" t="n">
+        <v>2</v>
+      </c>
+      <c r="T168" t="n">
         <v>5</v>
       </c>
-      <c r="E168" t="n">
-        <v>3</v>
-      </c>
-      <c r="F168" t="n">
-        <v>2</v>
-      </c>
-      <c r="G168" s="6" t="inlineStr">
-        <is>
-          <t>Low Cost</t>
-        </is>
-      </c>
-      <c r="H168" t="inlineStr"/>
-      <c r="I168" t="inlineStr"/>
-      <c r="J168" t="inlineStr"/>
-      <c r="K168" t="inlineStr"/>
-      <c r="L168" t="inlineStr"/>
-      <c r="M168" t="n">
-        <v>0</v>
-      </c>
-      <c r="N168" t="inlineStr"/>
-      <c r="O168" t="inlineStr"/>
-      <c r="P168" t="inlineStr"/>
-      <c r="Q168" t="inlineStr"/>
-      <c r="R168" t="inlineStr"/>
-      <c r="S168" t="n">
-        <v>2</v>
-      </c>
-      <c r="T168" t="n">
-        <v>6</v>
-      </c>
       <c r="U168" t="n">
         <v>0</v>
       </c>
       <c r="V168" t="n">
         <v>0</v>
       </c>
-      <c r="W168" t="inlineStr"/>
-      <c r="X168" t="inlineStr"/>
+      <c r="W168" t="n">
+        <v>1</v>
+      </c>
+      <c r="X168" t="n">
+        <v>0</v>
+      </c>
       <c r="Y168" t="inlineStr"/>
       <c r="Z168" t="inlineStr"/>
       <c r="AA168" t="inlineStr"/>
@@ -19563,7 +19565,7 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Bakoune</t>
+          <t>Sagrado</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
@@ -19573,11 +19575,11 @@
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>Monza</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E169" t="n">
         <v>4</v>
@@ -19590,33 +19592,57 @@
           <t>Low Cost</t>
         </is>
       </c>
-      <c r="H169" t="inlineStr"/>
-      <c r="I169" t="inlineStr"/>
-      <c r="J169" t="inlineStr"/>
-      <c r="K169" t="inlineStr"/>
-      <c r="L169" t="inlineStr"/>
+      <c r="H169" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="I169" t="inlineStr">
+        <is>
+          <t>Equo</t>
+        </is>
+      </c>
+      <c r="J169" t="n">
+        <v>3</v>
+      </c>
+      <c r="K169" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="L169" t="n">
+        <v>5.33</v>
+      </c>
       <c r="M169" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N169" t="inlineStr"/>
-      <c r="O169" t="inlineStr"/>
-      <c r="P169" t="inlineStr"/>
-      <c r="Q169" t="inlineStr"/>
-      <c r="R169" t="inlineStr"/>
+      <c r="O169" t="n">
+        <v>0.079</v>
+      </c>
+      <c r="P169" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q169" t="n">
+        <v>0</v>
+      </c>
+      <c r="R169" t="n">
+        <v>0</v>
+      </c>
       <c r="S169" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T169" t="n">
-        <v>6</v>
+        <v>7.5</v>
       </c>
       <c r="U169" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V169" t="n">
         <v>0</v>
       </c>
-      <c r="W169" t="inlineStr"/>
-      <c r="X169" t="inlineStr"/>
+      <c r="W169" t="n">
+        <v>1</v>
+      </c>
+      <c r="X169" t="n">
+        <v>0</v>
+      </c>
       <c r="Y169" t="inlineStr"/>
       <c r="Z169" t="inlineStr"/>
       <c r="AA169" t="inlineStr"/>
@@ -19624,24 +19650,24 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Terzic</t>
+          <t>Kofler</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Ds;E</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="D170" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E170" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F170" t="n">
         <v>2</v>
@@ -19668,7 +19694,7 @@
         <v>2</v>
       </c>
       <c r="T170" t="n">
-        <v>5.75</v>
+        <v>6</v>
       </c>
       <c r="U170" t="n">
         <v>0</v>
@@ -19685,27 +19711,27 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Mitaj</t>
+          <t>Bakoune</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Ds;E</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Monza</t>
         </is>
       </c>
       <c r="D171" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E171" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="F171" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G171" s="6" t="inlineStr">
         <is>
@@ -19726,10 +19752,10 @@
       <c r="Q171" t="inlineStr"/>
       <c r="R171" t="inlineStr"/>
       <c r="S171" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T171" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U171" t="n">
         <v>0</v>
@@ -19746,7 +19772,7 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Alhassane</t>
+          <t>Terzic</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
@@ -19756,17 +19782,17 @@
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>Bologna</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D172" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E172" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F172" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G172" s="6" t="inlineStr">
         <is>
@@ -19807,27 +19833,27 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Akpoguma</t>
+          <t>Alhassane</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Dc</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Bologna</t>
         </is>
       </c>
       <c r="D173" t="n">
         <v>2</v>
       </c>
       <c r="E173" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F173" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G173" s="6" t="inlineStr">
         <is>
@@ -19848,10 +19874,10 @@
       <c r="Q173" t="inlineStr"/>
       <c r="R173" t="inlineStr"/>
       <c r="S173" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T173" t="n">
-        <v>0</v>
+        <v>5.75</v>
       </c>
       <c r="U173" t="n">
         <v>0</v>
@@ -19868,24 +19894,24 @@
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Puczka</t>
+          <t>Akpoguma</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Ds;E</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D174" t="n">
         <v>2</v>
       </c>
       <c r="E174" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F174" t="n">
         <v>2</v>
@@ -19909,10 +19935,10 @@
       <c r="Q174" t="inlineStr"/>
       <c r="R174" t="inlineStr"/>
       <c r="S174" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T174" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="U174" t="n">
         <v>0</v>
@@ -19929,27 +19955,27 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>Halhal</t>
+          <t>Puczka</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Dc</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>Venezia</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="D175" t="n">
         <v>2</v>
       </c>
       <c r="E175" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F175" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G175" s="6" t="inlineStr">
         <is>
@@ -19970,10 +19996,10 @@
       <c r="Q175" t="inlineStr"/>
       <c r="R175" t="inlineStr"/>
       <c r="S175" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T175" t="n">
-        <v>3.5</v>
+        <v>6</v>
       </c>
       <c r="U175" t="n">
         <v>0</v>
@@ -19990,12 +20016,12 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Franjic</t>
+          <t>Halhal</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>B;Ds;E</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
@@ -20007,10 +20033,10 @@
         <v>2</v>
       </c>
       <c r="E176" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F176" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G176" s="6" t="inlineStr">
         <is>
@@ -20034,7 +20060,7 @@
         <v>2</v>
       </c>
       <c r="T176" t="n">
-        <v>5.75</v>
+        <v>3.5</v>
       </c>
       <c r="U176" t="n">
         <v>0</v>
@@ -20051,17 +20077,17 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Tchato</t>
+          <t>Franjic</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Dd;E</t>
+          <t>B;Ds;E</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>Frosinone</t>
+          <t>Venezia</t>
         </is>
       </c>
       <c r="D177" t="n">
@@ -20092,10 +20118,10 @@
       <c r="Q177" t="inlineStr"/>
       <c r="R177" t="inlineStr"/>
       <c r="S177" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T177" t="n">
-        <v>0</v>
+        <v>5.75</v>
       </c>
       <c r="U177" t="n">
         <v>0</v>
@@ -20112,27 +20138,27 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Kambwala</t>
+          <t>Tchato</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Dd;Dc</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Frosinone</t>
         </is>
       </c>
       <c r="D178" t="n">
         <v>2</v>
       </c>
       <c r="E178" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F178" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G178" s="6" t="inlineStr">
         <is>
@@ -20173,24 +20199,24 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Drameh</t>
+          <t>Kambwala</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Dd;Ds;E</t>
+          <t>Dd;Dc</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>Genoa</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="D179" t="n">
         <v>2</v>
       </c>
       <c r="E179" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F179" t="n">
         <v>2</v>
@@ -20234,24 +20260,24 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Diawara S.</t>
+          <t>Drameh</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Ds;Dc</t>
+          <t>Dd;Ds;E</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>Milan</t>
+          <t>Genoa</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E180" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F180" t="n">
         <v>2</v>
@@ -20295,17 +20321,17 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Aurelio</t>
+          <t>Diawara S.</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Ds;E</t>
+          <t>Ds;Dc</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>Cagliari</t>
+          <t>Milan</t>
         </is>
       </c>
       <c r="D181" t="n">
@@ -20356,68 +20382,46 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Dembelè A.</t>
+          <t>Aurelio</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Dd;E</t>
+          <t>Ds;E</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>Lecce</t>
+          <t>Cagliari</t>
         </is>
       </c>
       <c r="D182" t="n">
         <v>1</v>
       </c>
       <c r="E182" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F182" t="n">
-        <v>1</v>
-      </c>
-      <c r="G182" s="7" t="inlineStr">
-        <is>
-          <t>Scommessa</t>
-        </is>
-      </c>
-      <c r="H182" t="n">
-        <v>43.6</v>
-      </c>
-      <c r="I182" t="inlineStr">
-        <is>
-          <t>Affare</t>
-        </is>
-      </c>
-      <c r="J182" t="n">
-        <v>1</v>
-      </c>
-      <c r="K182" t="n">
-        <v>5</v>
-      </c>
-      <c r="L182" t="n">
-        <v>5</v>
-      </c>
+        <v>2</v>
+      </c>
+      <c r="G182" s="6" t="inlineStr">
+        <is>
+          <t>Low Cost</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr"/>
+      <c r="I182" t="inlineStr"/>
+      <c r="J182" t="inlineStr"/>
+      <c r="K182" t="inlineStr"/>
+      <c r="L182" t="inlineStr"/>
       <c r="M182" t="n">
-        <v>2</v>
-      </c>
-      <c r="N182" t="n">
-        <v>-0.89</v>
-      </c>
-      <c r="O182" t="n">
-        <v>0.132</v>
-      </c>
-      <c r="P182" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q182" t="n">
-        <v>0</v>
-      </c>
-      <c r="R182" t="n">
-        <v>0</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="N182" t="inlineStr"/>
+      <c r="O182" t="inlineStr"/>
+      <c r="P182" t="inlineStr"/>
+      <c r="Q182" t="inlineStr"/>
+      <c r="R182" t="inlineStr"/>
       <c r="S182" t="n">
         <v>0</v>
       </c>
@@ -20430,12 +20434,8 @@
       <c r="V182" t="n">
         <v>0</v>
       </c>
-      <c r="W182" t="n">
-        <v>0</v>
-      </c>
-      <c r="X182" t="n">
-        <v>0</v>
-      </c>
+      <c r="W182" t="inlineStr"/>
+      <c r="X182" t="inlineStr"/>
       <c r="Y182" t="inlineStr"/>
       <c r="Z182" t="inlineStr"/>
       <c r="AA182" t="inlineStr"/>
@@ -20443,24 +20443,24 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Goldaniga</t>
+          <t>Dembelè A.</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Dc</t>
+          <t>Dd;E</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>Como</t>
+          <t>Lecce</t>
         </is>
       </c>
       <c r="D183" t="n">
         <v>1</v>
       </c>
       <c r="E183" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F183" t="n">
         <v>1</v>
@@ -20471,7 +20471,7 @@
         </is>
       </c>
       <c r="H183" t="n">
-        <v>27</v>
+        <v>43.6</v>
       </c>
       <c r="I183" t="inlineStr">
         <is>
@@ -20479,22 +20479,22 @@
         </is>
       </c>
       <c r="J183" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="K183" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="L183" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="M183" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="N183" t="n">
-        <v>-5.66</v>
+        <v>-0.89</v>
       </c>
       <c r="O183" t="n">
-        <v>0.377</v>
+        <v>0.132</v>
       </c>
       <c r="P183" t="n">
         <v>0</v>
@@ -20530,27 +20530,27 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Carboni F.</t>
+          <t>Goldaniga</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Ds;E</t>
+          <t>Dc</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>Parma</t>
+          <t>Como</t>
         </is>
       </c>
       <c r="D184" t="n">
         <v>1</v>
       </c>
       <c r="E184" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F184" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G184" s="7" t="inlineStr">
         <is>
@@ -20558,30 +20558,30 @@
         </is>
       </c>
       <c r="H184" t="n">
-        <v>14.2</v>
+        <v>27</v>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>Equo</t>
+          <t>Affare</t>
         </is>
       </c>
       <c r="J184" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="K184" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="L184" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="M184" t="n">
         <v>3</v>
       </c>
       <c r="N184" t="n">
-        <v>2.44</v>
+        <v>-5.66</v>
       </c>
       <c r="O184" t="n">
-        <v>0.061</v>
+        <v>0.377</v>
       </c>
       <c r="P184" t="n">
         <v>0</v>
@@ -21113,8 +21113,69 @@
       <c r="Z191" t="inlineStr"/>
       <c r="AA191" t="inlineStr"/>
     </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>Obric</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>Dc</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Atalanta</t>
+        </is>
+      </c>
+      <c r="D192" t="n">
+        <v>1</v>
+      </c>
+      <c r="E192" t="n">
+        <v>1</v>
+      </c>
+      <c r="F192" t="n">
+        <v>1</v>
+      </c>
+      <c r="G192" s="7" t="inlineStr">
+        <is>
+          <t>Scommessa</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr"/>
+      <c r="I192" t="inlineStr"/>
+      <c r="J192" t="inlineStr"/>
+      <c r="K192" t="inlineStr"/>
+      <c r="L192" t="inlineStr"/>
+      <c r="M192" t="n">
+        <v>0</v>
+      </c>
+      <c r="N192" t="inlineStr"/>
+      <c r="O192" t="inlineStr"/>
+      <c r="P192" t="inlineStr"/>
+      <c r="Q192" t="inlineStr"/>
+      <c r="R192" t="inlineStr"/>
+      <c r="S192" t="n">
+        <v>0</v>
+      </c>
+      <c r="T192" t="n">
+        <v>0</v>
+      </c>
+      <c r="U192" t="n">
+        <v>0</v>
+      </c>
+      <c r="V192" t="n">
+        <v>0</v>
+      </c>
+      <c r="W192" t="inlineStr"/>
+      <c r="X192" t="inlineStr"/>
+      <c r="Y192" t="inlineStr"/>
+      <c r="Z192" t="inlineStr"/>
+      <c r="AA192" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:AA191"/>
+  <autoFilter ref="A1:AA192"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
chore: aggiornamento automatico dati fantacalcio 2026-10-06
</commit_message>
<xml_diff>
--- a/export/lista_asta.xlsx
+++ b/export/lista_asta.xlsx
@@ -24572,10 +24572,10 @@
         <v>11</v>
       </c>
       <c r="E41" t="n">
-        <v>32</v>
+        <v>20</v>
       </c>
       <c r="F41" t="n">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="G41" s="4" t="inlineStr">
         <is>
@@ -24587,7 +24587,7 @@
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>Equo</t>
+          <t>Affare</t>
         </is>
       </c>
       <c r="J41" t="n">

</xml_diff>

<commit_message>
chore: aggiornamento automatico dati fantacalcio 2026-10-18
</commit_message>
<xml_diff>
--- a/export/lista_asta.xlsx
+++ b/export/lista_asta.xlsx
@@ -878,7 +878,7 @@
         <v>0</v>
       </c>
       <c r="S4" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T4" t="n">
         <v>5</v>
@@ -965,10 +965,10 @@
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T5" t="n">
-        <v>4.67</v>
+        <v>4.71</v>
       </c>
       <c r="U5" t="n">
         <v>0</v>
@@ -1548,10 +1548,10 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T12" t="n">
-        <v>4.38</v>
+        <v>4.1</v>
       </c>
       <c r="U12" t="n">
         <v>0</v>
@@ -1809,10 +1809,10 @@
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T15" t="n">
-        <v>6.5</v>
+        <v>6.25</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -1894,10 +1894,10 @@
         <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T16" t="n">
-        <v>5.58</v>
+        <v>5.36</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
@@ -2301,10 +2301,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T21" t="n">
-        <v>3.42</v>
+        <v>4.5</v>
       </c>
       <c r="U21" t="n">
         <v>0</v>
@@ -2386,10 +2386,10 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T22" t="n">
-        <v>4</v>
+        <v>3.43</v>
       </c>
       <c r="U22" t="n">
         <v>0</v>
@@ -2558,7 +2558,7 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T24" t="n">
         <v>4</v>
@@ -6020,10 +6020,10 @@
         <v>0</v>
       </c>
       <c r="S2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T2" t="n">
-        <v>6.33</v>
+        <v>6.29</v>
       </c>
       <c r="U2" t="n">
         <v>0</v>
@@ -6366,10 +6366,10 @@
         <v>0</v>
       </c>
       <c r="S6" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T6" t="n">
-        <v>6.33</v>
+        <v>6.14</v>
       </c>
       <c r="U6" t="n">
         <v>0</v>
@@ -6688,10 +6688,10 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T10" t="n">
-        <v>5.9</v>
+        <v>5.83</v>
       </c>
       <c r="U10" t="n">
         <v>0</v>
@@ -6775,10 +6775,10 @@
         <v>0</v>
       </c>
       <c r="S11" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T11" t="n">
-        <v>6.58</v>
+        <v>6.5</v>
       </c>
       <c r="U11" t="n">
         <v>1</v>
@@ -6862,10 +6862,10 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T12" t="n">
-        <v>6.8</v>
+        <v>6.67</v>
       </c>
       <c r="U12" t="n">
         <v>1</v>
@@ -6949,10 +6949,10 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T13" t="n">
-        <v>6.17</v>
+        <v>6.07</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
@@ -7210,10 +7210,10 @@
         <v>0</v>
       </c>
       <c r="S16" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T16" t="n">
-        <v>5.58</v>
+        <v>5.5</v>
       </c>
       <c r="U16" t="n">
         <v>0</v>
@@ -7297,10 +7297,10 @@
         <v>0</v>
       </c>
       <c r="S17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T17" t="n">
-        <v>5.9</v>
+        <v>5.92</v>
       </c>
       <c r="U17" t="n">
         <v>0</v>
@@ -7382,10 +7382,10 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T18" t="n">
-        <v>5.8</v>
+        <v>5.83</v>
       </c>
       <c r="U18" t="n">
         <v>0</v>
@@ -7556,10 +7556,10 @@
         <v>0</v>
       </c>
       <c r="S20" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T20" t="n">
-        <v>5.75</v>
+        <v>5.8</v>
       </c>
       <c r="U20" t="n">
         <v>0</v>
@@ -7643,16 +7643,16 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T21" t="n">
-        <v>7.75</v>
+        <v>8.4</v>
       </c>
       <c r="U21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V21" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W21" t="n">
         <v>6</v>
@@ -7730,16 +7730,16 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T22" t="n">
-        <v>6.4</v>
+        <v>6.5</v>
       </c>
       <c r="U22" t="n">
         <v>0</v>
       </c>
       <c r="V22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W22" t="n">
         <v>6</v>
@@ -8707,7 +8707,7 @@
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T35" t="n">
         <v>6.5</v>
@@ -8964,10 +8964,10 @@
         <v>0</v>
       </c>
       <c r="S38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T38" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="U38" t="n">
         <v>0</v>
@@ -9136,10 +9136,10 @@
         <v>0</v>
       </c>
       <c r="S40" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T40" t="n">
-        <v>5.5</v>
+        <v>5.42</v>
       </c>
       <c r="U40" t="n">
         <v>1</v>
@@ -9310,10 +9310,10 @@
         <v>0</v>
       </c>
       <c r="S42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T42" t="n">
-        <v>6</v>
+        <v>5.83</v>
       </c>
       <c r="U42" t="n">
         <v>0</v>
@@ -10263,10 +10263,10 @@
         <v>0</v>
       </c>
       <c r="S53" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T53" t="n">
-        <v>7.33</v>
+        <v>7.14</v>
       </c>
       <c r="U53" t="n">
         <v>2</v>
@@ -11042,10 +11042,10 @@
         <v>0</v>
       </c>
       <c r="S62" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T62" t="n">
-        <v>5.33</v>
+        <v>5.36</v>
       </c>
       <c r="U62" t="n">
         <v>0</v>
@@ -11386,10 +11386,10 @@
         <v>0</v>
       </c>
       <c r="S66" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T66" t="n">
-        <v>6.58</v>
+        <v>6.36</v>
       </c>
       <c r="U66" t="n">
         <v>1</v>
@@ -11983,10 +11983,10 @@
         <v>0</v>
       </c>
       <c r="S73" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T73" t="n">
-        <v>6.42</v>
+        <v>6.43</v>
       </c>
       <c r="U73" t="n">
         <v>0</v>
@@ -12238,10 +12238,10 @@
         <v>0</v>
       </c>
       <c r="S76" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T76" t="n">
-        <v>6.12</v>
+        <v>6</v>
       </c>
       <c r="U76" t="n">
         <v>0</v>
@@ -12390,10 +12390,10 @@
       <c r="Q78" t="inlineStr"/>
       <c r="R78" t="inlineStr"/>
       <c r="S78" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T78" t="n">
-        <v>6.75</v>
+        <v>6.64</v>
       </c>
       <c r="U78" t="n">
         <v>1</v>
@@ -12573,10 +12573,10 @@
       <c r="Q81" t="inlineStr"/>
       <c r="R81" t="inlineStr"/>
       <c r="S81" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T81" t="n">
-        <v>5.83</v>
+        <v>5.75</v>
       </c>
       <c r="U81" t="n">
         <v>0</v>
@@ -12817,10 +12817,10 @@
       <c r="Q85" t="inlineStr"/>
       <c r="R85" t="inlineStr"/>
       <c r="S85" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T85" t="n">
-        <v>5.75</v>
+        <v>5.33</v>
       </c>
       <c r="U85" t="n">
         <v>0</v>
@@ -12939,13 +12939,13 @@
       <c r="Q87" t="inlineStr"/>
       <c r="R87" t="inlineStr"/>
       <c r="S87" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T87" t="n">
-        <v>6.25</v>
+        <v>7</v>
       </c>
       <c r="U87" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V87" t="n">
         <v>0</v>
@@ -13192,10 +13192,10 @@
         <v>0</v>
       </c>
       <c r="S90" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T90" t="n">
-        <v>6</v>
+        <v>5.9</v>
       </c>
       <c r="U90" t="n">
         <v>0</v>
@@ -13540,10 +13540,10 @@
         <v>0</v>
       </c>
       <c r="S94" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T94" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U94" t="n">
         <v>0</v>
@@ -13714,7 +13714,7 @@
         <v>0</v>
       </c>
       <c r="S96" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T96" t="n">
         <v>6</v>
@@ -14234,10 +14234,10 @@
         <v>0</v>
       </c>
       <c r="S102" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T102" t="n">
-        <v>5.62</v>
+        <v>5.8</v>
       </c>
       <c r="U102" t="n">
         <v>0</v>
@@ -15015,10 +15015,10 @@
         <v>0</v>
       </c>
       <c r="S111" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T111" t="n">
-        <v>5.5</v>
+        <v>5.25</v>
       </c>
       <c r="U111" t="n">
         <v>0</v>
@@ -15707,10 +15707,10 @@
         <v>0</v>
       </c>
       <c r="S119" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T119" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U119" t="n">
         <v>0</v>
@@ -16225,10 +16225,10 @@
         <v>0</v>
       </c>
       <c r="S125" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T125" t="n">
-        <v>5</v>
+        <v>5.5</v>
       </c>
       <c r="U125" t="n">
         <v>0</v>
@@ -16310,10 +16310,10 @@
         <v>0</v>
       </c>
       <c r="S126" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T126" t="n">
-        <v>5.67</v>
+        <v>5.79</v>
       </c>
       <c r="U126" t="n">
         <v>0</v>
@@ -16397,10 +16397,10 @@
         <v>0</v>
       </c>
       <c r="S127" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T127" t="n">
-        <v>6.5</v>
+        <v>6</v>
       </c>
       <c r="U127" t="n">
         <v>0</v>
@@ -16482,10 +16482,10 @@
         <v>0</v>
       </c>
       <c r="S128" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T128" t="n">
-        <v>5.1</v>
+        <v>5.25</v>
       </c>
       <c r="U128" t="n">
         <v>0</v>
@@ -16567,10 +16567,10 @@
         <v>0</v>
       </c>
       <c r="S129" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T129" t="n">
-        <v>4.88</v>
+        <v>5</v>
       </c>
       <c r="U129" t="n">
         <v>0</v>
@@ -16652,10 +16652,10 @@
         <v>0</v>
       </c>
       <c r="S130" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T130" t="n">
-        <v>10</v>
+        <v>8.33</v>
       </c>
       <c r="U130" t="n">
         <v>2</v>
@@ -17133,7 +17133,7 @@
       <c r="Q137" t="inlineStr"/>
       <c r="R137" t="inlineStr"/>
       <c r="S137" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T137" t="n">
         <v>6</v>
@@ -17255,10 +17255,10 @@
       <c r="Q139" t="inlineStr"/>
       <c r="R139" t="inlineStr"/>
       <c r="S139" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T139" t="n">
-        <v>5.25</v>
+        <v>5.33</v>
       </c>
       <c r="U139" t="n">
         <v>0</v>
@@ -17621,10 +17621,10 @@
       <c r="Q145" t="inlineStr"/>
       <c r="R145" t="inlineStr"/>
       <c r="S145" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T145" t="n">
-        <v>4</v>
+        <v>4.62</v>
       </c>
       <c r="U145" t="n">
         <v>0</v>
@@ -17702,7 +17702,7 @@
         <v>0</v>
       </c>
       <c r="S146" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T146" t="n">
         <v>6</v>
@@ -19998,10 +19998,10 @@
       <c r="Q174" t="inlineStr"/>
       <c r="R174" t="inlineStr"/>
       <c r="S174" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T174" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="U174" t="n">
         <v>0</v>
@@ -21270,10 +21270,10 @@
       <c r="Q192" t="inlineStr"/>
       <c r="R192" t="inlineStr"/>
       <c r="S192" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T192" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="U192" t="n">
         <v>0</v>
@@ -21769,10 +21769,10 @@
         <v>1</v>
       </c>
       <c r="S4" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T4" t="n">
-        <v>5.83</v>
+        <v>5.75</v>
       </c>
       <c r="U4" t="n">
         <v>0</v>
@@ -21856,10 +21856,10 @@
         <v>5</v>
       </c>
       <c r="S5" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T5" t="n">
-        <v>8.880000000000001</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="U5" t="n">
         <v>3</v>
@@ -22550,16 +22550,16 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T13" t="n">
-        <v>7</v>
+        <v>7.08</v>
       </c>
       <c r="U13" t="n">
         <v>1</v>
       </c>
       <c r="V13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W13" t="n">
         <v>7</v>
@@ -22983,10 +22983,10 @@
         <v>3</v>
       </c>
       <c r="S18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T18" t="n">
-        <v>8.25</v>
+        <v>7.36</v>
       </c>
       <c r="U18" t="n">
         <v>3</v>
@@ -23244,10 +23244,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T21" t="n">
-        <v>6.6</v>
+        <v>6.5</v>
       </c>
       <c r="U21" t="n">
         <v>1</v>
@@ -23416,16 +23416,16 @@
         <v>1</v>
       </c>
       <c r="S23" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T23" t="n">
-        <v>7.3</v>
+        <v>7.33</v>
       </c>
       <c r="U23" t="n">
         <v>1</v>
       </c>
       <c r="V23" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W23" t="n">
         <v>3</v>
@@ -23673,10 +23673,10 @@
         <v>1</v>
       </c>
       <c r="S26" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T26" t="n">
-        <v>7</v>
+        <v>6.75</v>
       </c>
       <c r="U26" t="n">
         <v>1</v>
@@ -24191,10 +24191,10 @@
         <v>0</v>
       </c>
       <c r="S32" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T32" t="n">
-        <v>7</v>
+        <v>6.92</v>
       </c>
       <c r="U32" t="n">
         <v>0</v>
@@ -24256,10 +24256,10 @@
       <c r="Q33" t="inlineStr"/>
       <c r="R33" t="inlineStr"/>
       <c r="S33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T33" t="n">
-        <v>7.12</v>
+        <v>6.9</v>
       </c>
       <c r="U33" t="n">
         <v>1</v>
@@ -24439,16 +24439,16 @@
       <c r="Q36" t="inlineStr"/>
       <c r="R36" t="inlineStr"/>
       <c r="S36" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T36" t="n">
-        <v>7.08</v>
+        <v>7.71</v>
       </c>
       <c r="U36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W36" t="inlineStr"/>
       <c r="X36" t="inlineStr"/>
@@ -24500,10 +24500,10 @@
       <c r="Q37" t="inlineStr"/>
       <c r="R37" t="inlineStr"/>
       <c r="S37" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T37" t="n">
-        <v>6.58</v>
+        <v>6.57</v>
       </c>
       <c r="U37" t="n">
         <v>0</v>
@@ -25197,13 +25197,13 @@
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T46" t="n">
-        <v>5.67</v>
+        <v>6.21</v>
       </c>
       <c r="U46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V46" t="n">
         <v>0</v>
@@ -25545,10 +25545,10 @@
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T50" t="n">
-        <v>6.33</v>
+        <v>6.29</v>
       </c>
       <c r="U50" t="n">
         <v>0</v>
@@ -25893,10 +25893,10 @@
         <v>0</v>
       </c>
       <c r="S54" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T54" t="n">
-        <v>7.62</v>
+        <v>7.3</v>
       </c>
       <c r="U54" t="n">
         <v>2</v>
@@ -26152,10 +26152,10 @@
         <v>0</v>
       </c>
       <c r="S57" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T57" t="n">
-        <v>6.9</v>
+        <v>6.67</v>
       </c>
       <c r="U57" t="n">
         <v>1</v>
@@ -26846,10 +26846,10 @@
         <v>0</v>
       </c>
       <c r="S65" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T65" t="n">
-        <v>5.83</v>
+        <v>5.79</v>
       </c>
       <c r="U65" t="n">
         <v>0</v>
@@ -27020,10 +27020,10 @@
         <v>0</v>
       </c>
       <c r="S67" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T67" t="n">
-        <v>6.17</v>
+        <v>6.07</v>
       </c>
       <c r="U67" t="n">
         <v>0</v>
@@ -27107,10 +27107,10 @@
         <v>0</v>
       </c>
       <c r="S68" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T68" t="n">
-        <v>6.58</v>
+        <v>6.43</v>
       </c>
       <c r="U68" t="n">
         <v>0</v>
@@ -27194,10 +27194,10 @@
         <v>0</v>
       </c>
       <c r="S69" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T69" t="n">
-        <v>6.92</v>
+        <v>6.79</v>
       </c>
       <c r="U69" t="n">
         <v>1</v>
@@ -27801,7 +27801,7 @@
         <v>0</v>
       </c>
       <c r="S76" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T76" t="n">
         <v>6.5</v>
@@ -27810,7 +27810,7 @@
         <v>0</v>
       </c>
       <c r="V76" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W76" t="n">
         <v>0</v>
@@ -28979,7 +28979,7 @@
         <v>0</v>
       </c>
       <c r="S92" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T92" t="n">
         <v>6.5</v>
@@ -29240,7 +29240,7 @@
         <v>2</v>
       </c>
       <c r="S95" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T95" t="n">
         <v>6</v>
@@ -29588,10 +29588,10 @@
         <v>0</v>
       </c>
       <c r="S99" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T99" t="n">
-        <v>6.17</v>
+        <v>6.12</v>
       </c>
       <c r="U99" t="n">
         <v>0</v>
@@ -29675,10 +29675,10 @@
         <v>1</v>
       </c>
       <c r="S100" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T100" t="n">
-        <v>6.75</v>
+        <v>6.57</v>
       </c>
       <c r="U100" t="n">
         <v>1</v>
@@ -30108,10 +30108,10 @@
         <v>0</v>
       </c>
       <c r="S105" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T105" t="n">
-        <v>5.83</v>
+        <v>5.75</v>
       </c>
       <c r="U105" t="n">
         <v>0</v>
@@ -30369,13 +30369,13 @@
         <v>0</v>
       </c>
       <c r="S108" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T108" t="n">
-        <v>6.2</v>
+        <v>6.75</v>
       </c>
       <c r="U108" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V108" t="n">
         <v>0</v>
@@ -30456,10 +30456,10 @@
         <v>0</v>
       </c>
       <c r="S109" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T109" t="n">
-        <v>5.88</v>
+        <v>5.9</v>
       </c>
       <c r="U109" t="n">
         <v>0</v>
@@ -30717,10 +30717,10 @@
         <v>0</v>
       </c>
       <c r="S112" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T112" t="n">
-        <v>5.67</v>
+        <v>5.57</v>
       </c>
       <c r="U112" t="n">
         <v>0</v>
@@ -30802,10 +30802,10 @@
         <v>0</v>
       </c>
       <c r="S113" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T113" t="n">
-        <v>6</v>
+        <v>5.8</v>
       </c>
       <c r="U113" t="n">
         <v>0</v>
@@ -31148,10 +31148,10 @@
         <v>0</v>
       </c>
       <c r="S117" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T117" t="n">
-        <v>5.83</v>
+        <v>5.75</v>
       </c>
       <c r="U117" t="n">
         <v>0</v>
@@ -31233,10 +31233,10 @@
         <v>0</v>
       </c>
       <c r="S118" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T118" t="n">
-        <v>5.67</v>
+        <v>5.71</v>
       </c>
       <c r="U118" t="n">
         <v>0</v>
@@ -31407,10 +31407,10 @@
         <v>0</v>
       </c>
       <c r="S120" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T120" t="n">
-        <v>7.33</v>
+        <v>7</v>
       </c>
       <c r="U120" t="n">
         <v>1</v>
@@ -31579,16 +31579,16 @@
         <v>0</v>
       </c>
       <c r="S122" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T122" t="n">
-        <v>5.4</v>
+        <v>5.75</v>
       </c>
       <c r="U122" t="n">
         <v>0</v>
       </c>
       <c r="V122" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W122" t="n">
         <v>3</v>
@@ -31840,10 +31840,10 @@
         <v>0</v>
       </c>
       <c r="S125" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T125" t="n">
-        <v>6.25</v>
+        <v>6.17</v>
       </c>
       <c r="U125" t="n">
         <v>0</v>
@@ -32184,10 +32184,10 @@
         <v>0</v>
       </c>
       <c r="S129" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T129" t="n">
-        <v>6.33</v>
+        <v>6.43</v>
       </c>
       <c r="U129" t="n">
         <v>0</v>
@@ -33963,10 +33963,10 @@
         <v>0</v>
       </c>
       <c r="S152" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T152" t="n">
-        <v>6.25</v>
+        <v>6.17</v>
       </c>
       <c r="U152" t="n">
         <v>0</v>
@@ -34137,10 +34137,10 @@
         <v>0</v>
       </c>
       <c r="S154" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T154" t="n">
-        <v>5.5</v>
+        <v>5.67</v>
       </c>
       <c r="U154" t="n">
         <v>0</v>
@@ -34746,10 +34746,10 @@
         <v>0</v>
       </c>
       <c r="S161" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T161" t="n">
-        <v>5.83</v>
+        <v>5.88</v>
       </c>
       <c r="U161" t="n">
         <v>0</v>
@@ -36471,7 +36471,7 @@
       <c r="Q184" t="inlineStr"/>
       <c r="R184" t="inlineStr"/>
       <c r="S184" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T184" t="n">
         <v>5.5</v>
@@ -37680,13 +37680,13 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T3" t="n">
-        <v>8.9</v>
+        <v>9</v>
       </c>
       <c r="U3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V3" t="n">
         <v>2</v>
@@ -37765,10 +37765,10 @@
         <v>1</v>
       </c>
       <c r="S4" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T4" t="n">
-        <v>7.17</v>
+        <v>7.07</v>
       </c>
       <c r="U4" t="n">
         <v>2</v>
@@ -38259,13 +38259,13 @@
         <v>3</v>
       </c>
       <c r="S10" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T10" t="n">
-        <v>6.5</v>
+        <v>7.08</v>
       </c>
       <c r="U10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V10" t="n">
         <v>0</v>
@@ -38431,10 +38431,10 @@
         <v>0</v>
       </c>
       <c r="S12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T12" t="n">
-        <v>8.199999999999999</v>
+        <v>7.67</v>
       </c>
       <c r="U12" t="n">
         <v>2</v>
@@ -38518,10 +38518,10 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T13" t="n">
-        <v>7.5</v>
+        <v>7.36</v>
       </c>
       <c r="U13" t="n">
         <v>2</v>
@@ -39186,10 +39186,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T21" t="n">
-        <v>6.42</v>
+        <v>6.29</v>
       </c>
       <c r="U21" t="n">
         <v>0</v>
@@ -39273,7 +39273,7 @@
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T22" t="n">
         <v>7.5</v>
@@ -39282,7 +39282,7 @@
         <v>1</v>
       </c>
       <c r="V22" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W22" t="n">
         <v>6</v>
@@ -39534,10 +39534,10 @@
         <v>0</v>
       </c>
       <c r="S25" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T25" t="n">
-        <v>6.67</v>
+        <v>6.38</v>
       </c>
       <c r="U25" t="n">
         <v>1</v>
@@ -39621,13 +39621,13 @@
         <v>0</v>
       </c>
       <c r="S26" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T26" t="n">
-        <v>6</v>
+        <v>6.8</v>
       </c>
       <c r="U26" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V26" t="n">
         <v>0</v>
@@ -39967,10 +39967,10 @@
         <v>0</v>
       </c>
       <c r="S30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T30" t="n">
-        <v>6</v>
+        <v>6.12</v>
       </c>
       <c r="U30" t="n">
         <v>0</v>
@@ -40054,10 +40054,10 @@
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T31" t="n">
-        <v>6.33</v>
+        <v>6.29</v>
       </c>
       <c r="U31" t="n">
         <v>1</v>
@@ -40226,10 +40226,10 @@
         <v>0</v>
       </c>
       <c r="S33" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T33" t="n">
-        <v>6.67</v>
+        <v>6.43</v>
       </c>
       <c r="U33" t="n">
         <v>1</v>
@@ -40398,10 +40398,10 @@
         <v>0</v>
       </c>
       <c r="S35" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T35" t="n">
-        <v>6.25</v>
+        <v>6.3</v>
       </c>
       <c r="U35" t="n">
         <v>0</v>
@@ -40483,10 +40483,10 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T36" t="n">
-        <v>8.33</v>
+        <v>8.140000000000001</v>
       </c>
       <c r="U36" t="n">
         <v>3</v>
@@ -40655,13 +40655,13 @@
         <v>0</v>
       </c>
       <c r="S38" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T38" t="n">
-        <v>8.25</v>
+        <v>9.57</v>
       </c>
       <c r="U38" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="V38" t="n">
         <v>0</v>
@@ -40842,10 +40842,10 @@
       <c r="Q41" t="inlineStr"/>
       <c r="R41" t="inlineStr"/>
       <c r="S41" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T41" t="n">
-        <v>8.300000000000001</v>
+        <v>7.83</v>
       </c>
       <c r="U41" t="n">
         <v>3</v>
@@ -40903,13 +40903,13 @@
       <c r="Q42" t="inlineStr"/>
       <c r="R42" t="inlineStr"/>
       <c r="S42" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T42" t="n">
-        <v>6.08</v>
+        <v>6.64</v>
       </c>
       <c r="U42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V42" t="n">
         <v>0</v>
@@ -41073,13 +41073,13 @@
         <v>0</v>
       </c>
       <c r="S44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T44" t="n">
-        <v>7.33</v>
+        <v>8</v>
       </c>
       <c r="U44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V44" t="n">
         <v>0</v>
@@ -41506,7 +41506,7 @@
         <v>0</v>
       </c>
       <c r="S49" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T49" t="n">
         <v>5.5</v>
@@ -41678,10 +41678,10 @@
         <v>0</v>
       </c>
       <c r="S51" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T51" t="n">
-        <v>5.7</v>
+        <v>5.58</v>
       </c>
       <c r="U51" t="n">
         <v>0</v>
@@ -42020,10 +42020,10 @@
         <v>0</v>
       </c>
       <c r="S55" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T55" t="n">
-        <v>5.92</v>
+        <v>5.93</v>
       </c>
       <c r="U55" t="n">
         <v>1</v>
@@ -42856,10 +42856,10 @@
       <c r="Q67" t="inlineStr"/>
       <c r="R67" t="inlineStr"/>
       <c r="S67" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T67" t="n">
-        <v>5.5</v>
+        <v>5.67</v>
       </c>
       <c r="U67" t="n">
         <v>0</v>
@@ -42917,10 +42917,10 @@
       <c r="Q68" t="inlineStr"/>
       <c r="R68" t="inlineStr"/>
       <c r="S68" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T68" t="n">
-        <v>10</v>
+        <v>7.75</v>
       </c>
       <c r="U68" t="n">
         <v>1</v>
@@ -43085,10 +43085,10 @@
         <v>0</v>
       </c>
       <c r="S70" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T70" t="n">
-        <v>7.5</v>
+        <v>6.5</v>
       </c>
       <c r="U70" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
chore: aggiornamento automatico dati fantacalcio 2026-10-28
</commit_message>
<xml_diff>
--- a/export/lista_asta.xlsx
+++ b/export/lista_asta.xlsx
@@ -965,10 +965,10 @@
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T5" t="n">
-        <v>6.25</v>
+        <v>6</v>
       </c>
       <c r="U5" t="n">
         <v>0</v>
@@ -1635,10 +1635,10 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T13" t="n">
-        <v>5.25</v>
+        <v>4.94</v>
       </c>
       <c r="U13" t="n">
         <v>0</v>
@@ -1809,10 +1809,10 @@
         <v>0</v>
       </c>
       <c r="S15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T15" t="n">
-        <v>5.33</v>
+        <v>5.25</v>
       </c>
       <c r="U15" t="n">
         <v>0</v>
@@ -1959,10 +1959,10 @@
       <c r="Q17" t="inlineStr"/>
       <c r="R17" t="inlineStr"/>
       <c r="S17" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T17" t="n">
-        <v>4.83</v>
+        <v>4.57</v>
       </c>
       <c r="U17" t="n">
         <v>0</v>
@@ -3056,10 +3056,10 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T30" t="n">
-        <v>5</v>
+        <v>5.5</v>
       </c>
       <c r="U30" t="n">
         <v>0</v>
@@ -3494,10 +3494,10 @@
         <v>0</v>
       </c>
       <c r="S36" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T36" t="n">
-        <v>4</v>
+        <v>5.5</v>
       </c>
       <c r="U36" t="n">
         <v>0</v>
@@ -6107,10 +6107,10 @@
         <v>0</v>
       </c>
       <c r="S3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T3" t="n">
-        <v>6.29</v>
+        <v>6.19</v>
       </c>
       <c r="U3" t="n">
         <v>0</v>
@@ -6279,10 +6279,10 @@
         <v>0</v>
       </c>
       <c r="S5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T5" t="n">
-        <v>6.75</v>
+        <v>6.64</v>
       </c>
       <c r="U5" t="n">
         <v>0</v>
@@ -6540,10 +6540,10 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T8" t="n">
-        <v>7.43</v>
+        <v>7.31</v>
       </c>
       <c r="U8" t="n">
         <v>1</v>
@@ -7408,10 +7408,10 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T18" t="n">
-        <v>5.83</v>
+        <v>5.86</v>
       </c>
       <c r="U18" t="n">
         <v>0</v>
@@ -7667,10 +7667,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T21" t="n">
-        <v>7.17</v>
+        <v>7</v>
       </c>
       <c r="U21" t="n">
         <v>1</v>
@@ -7752,13 +7752,13 @@
         <v>0</v>
       </c>
       <c r="S22" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T22" t="n">
-        <v>6.69</v>
+        <v>7</v>
       </c>
       <c r="U22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V22" t="n">
         <v>0</v>
@@ -7926,10 +7926,10 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T24" t="n">
-        <v>6.4</v>
+        <v>6.25</v>
       </c>
       <c r="U24" t="n">
         <v>0</v>
@@ -8426,16 +8426,16 @@
       <c r="Q30" t="inlineStr"/>
       <c r="R30" t="inlineStr"/>
       <c r="S30" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T30" t="n">
-        <v>6.33</v>
+        <v>6.5</v>
       </c>
       <c r="U30" t="n">
         <v>0</v>
       </c>
       <c r="V30" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W30" t="inlineStr"/>
       <c r="X30" t="inlineStr"/>
@@ -8487,10 +8487,10 @@
       <c r="Q31" t="inlineStr"/>
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T31" t="n">
-        <v>7.2</v>
+        <v>7.08</v>
       </c>
       <c r="U31" t="n">
         <v>1</v>
@@ -8731,16 +8731,16 @@
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T35" t="n">
-        <v>5.93</v>
+        <v>6.12</v>
       </c>
       <c r="U35" t="n">
         <v>0</v>
       </c>
       <c r="V35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W35" t="inlineStr"/>
       <c r="X35" t="inlineStr"/>
@@ -8988,10 +8988,10 @@
         <v>0</v>
       </c>
       <c r="S38" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T38" t="n">
-        <v>6.38</v>
+        <v>6.3</v>
       </c>
       <c r="U38" t="n">
         <v>0</v>
@@ -9508,10 +9508,10 @@
         <v>0</v>
       </c>
       <c r="S44" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T44" t="n">
-        <v>5.62</v>
+        <v>5.5</v>
       </c>
       <c r="U44" t="n">
         <v>0</v>
@@ -9595,10 +9595,10 @@
         <v>0</v>
       </c>
       <c r="S45" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T45" t="n">
-        <v>5.83</v>
+        <v>5.62</v>
       </c>
       <c r="U45" t="n">
         <v>0</v>
@@ -10463,10 +10463,10 @@
         <v>0</v>
       </c>
       <c r="S55" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T55" t="n">
-        <v>6.06</v>
+        <v>5.94</v>
       </c>
       <c r="U55" t="n">
         <v>0</v>
@@ -10983,16 +10983,16 @@
         <v>0</v>
       </c>
       <c r="S61" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T61" t="n">
-        <v>5.56</v>
+        <v>5.67</v>
       </c>
       <c r="U61" t="n">
         <v>0</v>
       </c>
       <c r="V61" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W61" t="n">
         <v>8</v>
@@ -11070,10 +11070,10 @@
         <v>0</v>
       </c>
       <c r="S62" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T62" t="n">
-        <v>6.21</v>
+        <v>6.12</v>
       </c>
       <c r="U62" t="n">
         <v>1</v>
@@ -11501,10 +11501,10 @@
         <v>0</v>
       </c>
       <c r="S67" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T67" t="n">
-        <v>6.31</v>
+        <v>6.22</v>
       </c>
       <c r="U67" t="n">
         <v>1</v>
@@ -11586,13 +11586,13 @@
         <v>0</v>
       </c>
       <c r="S68" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T68" t="n">
-        <v>5.81</v>
+        <v>6.28</v>
       </c>
       <c r="U68" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V68" t="n">
         <v>0</v>
@@ -11671,10 +11671,10 @@
         <v>0</v>
       </c>
       <c r="S69" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T69" t="n">
-        <v>5.69</v>
+        <v>5.61</v>
       </c>
       <c r="U69" t="n">
         <v>0</v>
@@ -12100,10 +12100,10 @@
         <v>0</v>
       </c>
       <c r="S74" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T74" t="n">
-        <v>5.88</v>
+        <v>5.78</v>
       </c>
       <c r="U74" t="n">
         <v>0</v>
@@ -12753,10 +12753,10 @@
       <c r="Q83" t="inlineStr"/>
       <c r="R83" t="inlineStr"/>
       <c r="S83" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T83" t="n">
-        <v>6.1</v>
+        <v>5.67</v>
       </c>
       <c r="U83" t="n">
         <v>0</v>
@@ -12875,16 +12875,16 @@
       <c r="Q85" t="inlineStr"/>
       <c r="R85" t="inlineStr"/>
       <c r="S85" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T85" t="n">
-        <v>7</v>
+        <v>7.75</v>
       </c>
       <c r="U85" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V85" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W85" t="inlineStr"/>
       <c r="X85" t="inlineStr"/>
@@ -12936,10 +12936,10 @@
       <c r="Q86" t="inlineStr"/>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T86" t="n">
-        <v>5.25</v>
+        <v>4.9</v>
       </c>
       <c r="U86" t="n">
         <v>0</v>
@@ -14553,10 +14553,10 @@
         <v>0</v>
       </c>
       <c r="S105" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T105" t="n">
-        <v>5.86</v>
+        <v>5.75</v>
       </c>
       <c r="U105" t="n">
         <v>0</v>
@@ -15848,16 +15848,16 @@
         <v>0</v>
       </c>
       <c r="S120" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T120" t="n">
-        <v>6</v>
+        <v>6.38</v>
       </c>
       <c r="U120" t="n">
         <v>0</v>
       </c>
       <c r="V120" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W120" t="n">
         <v>1</v>
@@ -16617,10 +16617,10 @@
         <v>0</v>
       </c>
       <c r="S129" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T129" t="n">
-        <v>8.33</v>
+        <v>7.25</v>
       </c>
       <c r="U129" t="n">
         <v>2</v>
@@ -16915,10 +16915,10 @@
       <c r="Q133" t="inlineStr"/>
       <c r="R133" t="inlineStr"/>
       <c r="S133" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T133" t="n">
-        <v>6.38</v>
+        <v>6.3</v>
       </c>
       <c r="U133" t="n">
         <v>0</v>
@@ -17159,10 +17159,10 @@
       <c r="Q137" t="inlineStr"/>
       <c r="R137" t="inlineStr"/>
       <c r="S137" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T137" t="n">
-        <v>5.8</v>
+        <v>5.58</v>
       </c>
       <c r="U137" t="n">
         <v>0</v>
@@ -17220,10 +17220,10 @@
       <c r="Q138" t="inlineStr"/>
       <c r="R138" t="inlineStr"/>
       <c r="S138" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T138" t="n">
-        <v>5.75</v>
+        <v>5.67</v>
       </c>
       <c r="U138" t="n">
         <v>0</v>
@@ -17281,7 +17281,7 @@
       <c r="Q139" t="inlineStr"/>
       <c r="R139" t="inlineStr"/>
       <c r="S139" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T139" t="n">
         <v>6</v>
@@ -17586,16 +17586,16 @@
       <c r="Q144" t="inlineStr"/>
       <c r="R144" t="inlineStr"/>
       <c r="S144" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T144" t="n">
-        <v>6.1</v>
+        <v>6.08</v>
       </c>
       <c r="U144" t="n">
         <v>0</v>
       </c>
       <c r="V144" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W144" t="inlineStr"/>
       <c r="X144" t="inlineStr"/>
@@ -18679,7 +18679,7 @@
         <v>0</v>
       </c>
       <c r="S157" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T157" t="n">
         <v>6</v>
@@ -19902,7 +19902,7 @@
       <c r="Q172" t="inlineStr"/>
       <c r="R172" t="inlineStr"/>
       <c r="S172" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="T172" t="n">
         <v>5</v>
@@ -20828,10 +20828,10 @@
         <v>0</v>
       </c>
       <c r="S186" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T186" t="n">
-        <v>5</v>
+        <v>5.25</v>
       </c>
       <c r="U186" t="n">
         <v>0</v>
@@ -21595,16 +21595,16 @@
         <v>2</v>
       </c>
       <c r="S2" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T2" t="n">
-        <v>7.43</v>
+        <v>7.94</v>
       </c>
       <c r="U2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W2" t="n">
         <v>5</v>
@@ -22115,13 +22115,13 @@
         <v>0</v>
       </c>
       <c r="S8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T8" t="n">
-        <v>6.79</v>
+        <v>7.19</v>
       </c>
       <c r="U8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V8" t="n">
         <v>0</v>
@@ -22202,16 +22202,16 @@
         <v>1</v>
       </c>
       <c r="S9" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T9" t="n">
-        <v>6.88</v>
+        <v>7.17</v>
       </c>
       <c r="U9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V9" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="W9" t="n">
         <v>6</v>
@@ -22289,10 +22289,10 @@
         <v>0</v>
       </c>
       <c r="S10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T10" t="n">
-        <v>7.56</v>
+        <v>7.06</v>
       </c>
       <c r="U10" t="n">
         <v>3</v>
@@ -22376,10 +22376,10 @@
         <v>4</v>
       </c>
       <c r="S11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T11" t="n">
-        <v>6.19</v>
+        <v>6.22</v>
       </c>
       <c r="U11" t="n">
         <v>0</v>
@@ -22463,10 +22463,10 @@
         <v>5</v>
       </c>
       <c r="S12" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T12" t="n">
-        <v>6.25</v>
+        <v>6.17</v>
       </c>
       <c r="U12" t="n">
         <v>1</v>
@@ -23760,16 +23760,16 @@
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T27" t="n">
-        <v>7</v>
+        <v>7.62</v>
       </c>
       <c r="U27" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V27" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W27" t="n">
         <v>0</v>
@@ -23932,16 +23932,16 @@
         <v>0</v>
       </c>
       <c r="S29" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T29" t="n">
-        <v>6.62</v>
+        <v>7.11</v>
       </c>
       <c r="U29" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V29" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W29" t="n">
         <v>5</v>
@@ -24430,13 +24430,13 @@
       <c r="Q35" t="inlineStr"/>
       <c r="R35" t="inlineStr"/>
       <c r="S35" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T35" t="n">
-        <v>6.75</v>
+        <v>7.29</v>
       </c>
       <c r="U35" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V35" t="n">
         <v>0</v>
@@ -25249,10 +25249,10 @@
         <v>0</v>
       </c>
       <c r="S46" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T46" t="n">
-        <v>6.21</v>
+        <v>5.94</v>
       </c>
       <c r="U46" t="n">
         <v>1</v>
@@ -25336,10 +25336,10 @@
         <v>0</v>
       </c>
       <c r="S47" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T47" t="n">
-        <v>6.5</v>
+        <v>6.43</v>
       </c>
       <c r="U47" t="n">
         <v>0</v>
@@ -25597,10 +25597,10 @@
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T50" t="n">
-        <v>6.12</v>
+        <v>6</v>
       </c>
       <c r="U50" t="n">
         <v>0</v>
@@ -25684,10 +25684,10 @@
         <v>0</v>
       </c>
       <c r="S51" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T51" t="n">
-        <v>6.17</v>
+        <v>6.14</v>
       </c>
       <c r="U51" t="n">
         <v>0</v>
@@ -25858,13 +25858,13 @@
         <v>0</v>
       </c>
       <c r="S53" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T53" t="n">
-        <v>7</v>
+        <v>7.36</v>
       </c>
       <c r="U53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="V53" t="n">
         <v>0</v>
@@ -27679,10 +27679,10 @@
         <v>0</v>
       </c>
       <c r="S74" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T74" t="n">
-        <v>6.36</v>
+        <v>6.25</v>
       </c>
       <c r="U74" t="n">
         <v>0</v>
@@ -27764,10 +27764,10 @@
         <v>0</v>
       </c>
       <c r="S75" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T75" t="n">
-        <v>6.12</v>
+        <v>6.11</v>
       </c>
       <c r="U75" t="n">
         <v>0</v>
@@ -28175,10 +28175,10 @@
       <c r="Q80" t="inlineStr"/>
       <c r="R80" t="inlineStr"/>
       <c r="S80" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T80" t="n">
-        <v>6.62</v>
+        <v>6.5</v>
       </c>
       <c r="U80" t="n">
         <v>1</v>
@@ -28419,10 +28419,10 @@
       <c r="Q84" t="inlineStr"/>
       <c r="R84" t="inlineStr"/>
       <c r="S84" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T84" t="n">
-        <v>6.75</v>
+        <v>6.57</v>
       </c>
       <c r="U84" t="n">
         <v>1</v>
@@ -28480,10 +28480,10 @@
       <c r="Q85" t="inlineStr"/>
       <c r="R85" t="inlineStr"/>
       <c r="S85" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T85" t="n">
-        <v>6.3</v>
+        <v>6.33</v>
       </c>
       <c r="U85" t="n">
         <v>0</v>
@@ -28541,16 +28541,16 @@
       <c r="Q86" t="inlineStr"/>
       <c r="R86" t="inlineStr"/>
       <c r="S86" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T86" t="n">
-        <v>6.67</v>
+        <v>6.79</v>
       </c>
       <c r="U86" t="n">
         <v>1</v>
       </c>
       <c r="V86" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W86" t="inlineStr"/>
       <c r="X86" t="inlineStr"/>
@@ -29527,10 +29527,10 @@
         <v>0</v>
       </c>
       <c r="S98" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T98" t="n">
-        <v>6.7</v>
+        <v>6.58</v>
       </c>
       <c r="U98" t="n">
         <v>1</v>
@@ -29612,10 +29612,10 @@
         <v>0</v>
       </c>
       <c r="S99" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T99" t="n">
-        <v>6.5</v>
+        <v>6.25</v>
       </c>
       <c r="U99" t="n">
         <v>0</v>
@@ -29873,7 +29873,7 @@
         <v>0</v>
       </c>
       <c r="S102" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T102" t="n">
         <v>6</v>
@@ -30306,10 +30306,10 @@
         <v>0</v>
       </c>
       <c r="S107" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T107" t="n">
-        <v>5.75</v>
+        <v>5.71</v>
       </c>
       <c r="U107" t="n">
         <v>0</v>
@@ -31431,10 +31431,10 @@
         <v>0</v>
       </c>
       <c r="S120" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T120" t="n">
-        <v>6.12</v>
+        <v>6.06</v>
       </c>
       <c r="U120" t="n">
         <v>0</v>
@@ -31951,7 +31951,7 @@
         <v>0</v>
       </c>
       <c r="S126" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T126" t="n">
         <v>6</v>
@@ -32210,10 +32210,10 @@
         <v>0</v>
       </c>
       <c r="S129" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T129" t="n">
-        <v>5.57</v>
+        <v>5.62</v>
       </c>
       <c r="U129" t="n">
         <v>0</v>
@@ -32469,10 +32469,10 @@
         <v>0</v>
       </c>
       <c r="S132" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T132" t="n">
-        <v>6.29</v>
+        <v>6.38</v>
       </c>
       <c r="U132" t="n">
         <v>0</v>
@@ -34052,16 +34052,16 @@
         <v>0</v>
       </c>
       <c r="S153" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T153" t="n">
-        <v>6.88</v>
+        <v>7</v>
       </c>
       <c r="U153" t="n">
         <v>1</v>
       </c>
       <c r="V153" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="W153" t="n">
         <v>0</v>
@@ -34226,10 +34226,10 @@
         <v>0</v>
       </c>
       <c r="S155" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T155" t="n">
-        <v>6</v>
+        <v>5.5</v>
       </c>
       <c r="U155" t="n">
         <v>0</v>
@@ -34831,10 +34831,10 @@
         <v>0</v>
       </c>
       <c r="S162" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T162" t="n">
-        <v>5.8</v>
+        <v>5.5</v>
       </c>
       <c r="U162" t="n">
         <v>0</v>
@@ -37850,13 +37850,13 @@
         <v>4</v>
       </c>
       <c r="S5" t="n">
+        <v>8</v>
+      </c>
+      <c r="T5" t="n">
+        <v>9.119999999999999</v>
+      </c>
+      <c r="U5" t="n">
         <v>7</v>
-      </c>
-      <c r="T5" t="n">
-        <v>9</v>
-      </c>
-      <c r="U5" t="n">
-        <v>6</v>
       </c>
       <c r="V5" t="n">
         <v>1</v>
@@ -38259,10 +38259,10 @@
         <v>3</v>
       </c>
       <c r="S10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="T10" t="n">
-        <v>6.79</v>
+        <v>6.5</v>
       </c>
       <c r="U10" t="n">
         <v>2</v>
@@ -38346,10 +38346,10 @@
         <v>1</v>
       </c>
       <c r="S11" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T11" t="n">
-        <v>8.25</v>
+        <v>7.94</v>
       </c>
       <c r="U11" t="n">
         <v>5</v>
@@ -38518,10 +38518,10 @@
         <v>0</v>
       </c>
       <c r="S13" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T13" t="n">
-        <v>7.69</v>
+        <v>7.5</v>
       </c>
       <c r="U13" t="n">
         <v>3</v>
@@ -38951,10 +38951,10 @@
         <v>0</v>
       </c>
       <c r="S18" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T18" t="n">
-        <v>7</v>
+        <v>6.94</v>
       </c>
       <c r="U18" t="n">
         <v>2</v>
@@ -39186,10 +39186,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T21" t="n">
-        <v>6.19</v>
+        <v>6.11</v>
       </c>
       <c r="U21" t="n">
         <v>0</v>
@@ -39273,13 +39273,13 @@
         <v>1</v>
       </c>
       <c r="S22" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T22" t="n">
-        <v>7.5</v>
+        <v>8</v>
       </c>
       <c r="U22" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="V22" t="n">
         <v>1</v>
@@ -39360,10 +39360,10 @@
         <v>1</v>
       </c>
       <c r="S23" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="T23" t="n">
-        <v>6.88</v>
+        <v>6.7</v>
       </c>
       <c r="U23" t="n">
         <v>1</v>
@@ -39447,13 +39447,13 @@
         <v>0</v>
       </c>
       <c r="S24" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T24" t="n">
-        <v>8.08</v>
+        <v>8.359999999999999</v>
       </c>
       <c r="U24" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="V24" t="n">
         <v>0</v>
@@ -39708,10 +39708,10 @@
         <v>0</v>
       </c>
       <c r="S27" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T27" t="n">
-        <v>6.75</v>
+        <v>6.57</v>
       </c>
       <c r="U27" t="n">
         <v>1</v>
@@ -40056,13 +40056,13 @@
         <v>0</v>
       </c>
       <c r="S31" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="T31" t="n">
-        <v>7.75</v>
+        <v>8.640000000000001</v>
       </c>
       <c r="U31" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V31" t="n">
         <v>2</v>
@@ -40230,13 +40230,13 @@
         <v>0</v>
       </c>
       <c r="S33" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T33" t="n">
-        <v>7.69</v>
+        <v>7.94</v>
       </c>
       <c r="U33" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="V33" t="n">
         <v>0</v>
@@ -41591,10 +41591,10 @@
         <v>0</v>
       </c>
       <c r="S50" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T50" t="n">
-        <v>6.25</v>
+        <v>6.17</v>
       </c>
       <c r="U50" t="n">
         <v>1</v>
@@ -41765,13 +41765,13 @@
         <v>3</v>
       </c>
       <c r="S52" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="T52" t="n">
-        <v>5.5</v>
+        <v>7</v>
       </c>
       <c r="U52" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V52" t="n">
         <v>0</v>
@@ -42022,10 +42022,10 @@
         <v>0</v>
       </c>
       <c r="S55" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="T55" t="n">
-        <v>6.69</v>
+        <v>6.61</v>
       </c>
       <c r="U55" t="n">
         <v>1</v>
@@ -42366,10 +42366,10 @@
         <v>0</v>
       </c>
       <c r="S59" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="T59" t="n">
-        <v>7.4</v>
+        <v>7.08</v>
       </c>
       <c r="U59" t="n">
         <v>2</v>

</xml_diff>